<commit_message>
chore(work-log): refresh qa nexus work log with day 7 + m0 close totals
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -31,10 +31,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="32">
     <font>
@@ -2755,35 +2756,35 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="56" t="inlineStr">
         <is>
           <t>This workbook merges QA_Nexus_Work_Hours_Log.xlsx + Token_Savings_Log.xlsx into a single master.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="56" t="inlineStr">
         <is>
           <t>Token sheets are prefixed 'Tokens —' (Sessions / Daily Rollup / Per-Chat Comparison).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="56" t="inlineStr">
         <is>
           <t>Old Token_Savings_Log.xlsx deleted. Source-of-truth path is now docs/observability/QA_Nexus_Work_Log.xlsx in the project repo.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="56" t="inlineStr">
         <is>
           <t>Days 2-4 entries in 'Development' + 'All Sessions' are EOD-aggregate placeholders — refine to per-session granularity using the existing Day 0/1 row format if/when needed.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="56" t="inlineStr">
         <is>
           <t>Aggregator: scripts/update-work-log.py (auto-roll new sessions; see script header for usage).</t>
         </is>
@@ -3825,7 +3826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="56" min="1" max="1"/>
@@ -3852,6 +3853,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="57">
       <c r="A4" s="78" t="inlineStr">
         <is>
@@ -5654,25 +5656,61 @@
       </c>
       <c r="H59" s="108" t="n"/>
     </row>
-    <row r="60" ht="15" customHeight="1" s="57">
-      <c r="A60" s="106" t="inlineStr">
+    <row r="60" ht="64" customHeight="1" s="57">
+      <c r="A60" s="131" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B60" s="123" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C60" s="124" t="inlineStr">
+        <is>
+          <t>12:00 – 22:30</t>
+        </is>
+      </c>
+      <c r="D60" s="125" t="n">
+        <v>7</v>
+      </c>
+      <c r="E60" s="123" t="n">
+        <v>80</v>
+      </c>
+      <c r="F60" s="124" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="G60" s="124" t="inlineStr">
+        <is>
+          <t>M0 close ceremony</t>
+        </is>
+      </c>
+      <c r="H60" s="124" t="inlineStr">
+        <is>
+          <t>M0 close ceremony — Steps A-I + Step E. PRs #21+#22+#23+#24 squash-merged; PR #25 (FE M2) opened as Draft. Followups (t) closed via PR #24, (u)+(v) filed. CLAUDE.md Hard Rule #3 updated for 3-folder frame inventory post Claude Design v2 supersede. M0 completion report at docs/milestones/M0_completion_report.md. 4th halt-to-root-cause pattern codified (refined pre-merge gate: compare PR vs main, only NEW failures gate). 102 commits over M0 window, 17 PASS / 0 FAIL / 2 DEFERRED to M1.5. Final main HEAD 44b06ef.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="106" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B60" s="93" t="n"/>
-      <c r="C60" s="64" t="n"/>
-      <c r="D60" s="89">
+      <c r="B61" s="93" t="n"/>
+      <c r="C61" s="64" t="n"/>
+      <c r="D61" s="89">
         <f>SUM(D5:D59)</f>
         <v/>
       </c>
-      <c r="E60" s="88">
+      <c r="E61" s="88">
         <f>SUM(E5:E59)</f>
         <v/>
       </c>
-      <c r="F60" s="97" t="n"/>
-      <c r="G60" s="97" t="n"/>
-      <c r="H60" s="97" t="n"/>
+      <c r="F61" s="97" t="n"/>
+      <c r="G61" s="97" t="n"/>
+      <c r="H61" s="97" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -8798,7 +8836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="56" min="1" max="1"/>
@@ -8823,6 +8861,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="57">
       <c r="A4" s="78" t="inlineStr">
         <is>
@@ -9317,24 +9356,55 @@
       <c r="F23" s="112" t="n"/>
       <c r="G23" s="112" t="n"/>
     </row>
-    <row r="24" ht="15" customHeight="1" s="57">
-      <c r="A24" s="106" t="inlineStr">
+    <row r="24" ht="64" customHeight="1" s="57">
+      <c r="A24" s="131" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B24" s="123" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C24" s="124" t="inlineStr">
+        <is>
+          <t>12:00 – 22:30</t>
+        </is>
+      </c>
+      <c r="D24" s="125" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" s="123" t="n">
+        <v>80</v>
+      </c>
+      <c r="F24" s="124" t="inlineStr">
+        <is>
+          <t>M0 close ceremony</t>
+        </is>
+      </c>
+      <c r="G24" s="124" t="inlineStr">
+        <is>
+          <t>M0 close ceremony — Steps A-I + Step E. PRs #21+#22+#23+#24 squash-merged; PR #25 (FE M2) opened as Draft. Followups (t) closed via PR #24, (u)+(v) filed. CLAUDE.md Hard Rule #3 updated for 3-folder frame inventory post Claude Design v2 supersede. M0 completion report at docs/milestones/M0_completion_report.md. 4th halt-to-root-cause pattern codified (refined pre-merge gate: compare PR vs main, only NEW failures gate). 102 commits over M0 window, 17 PASS / 0 FAIL / 2 DEFERRED to M1.5. Final main HEAD 44b06ef.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="106" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B24" s="93" t="n"/>
-      <c r="C24" s="64" t="n"/>
-      <c r="D24" s="89">
+      <c r="B25" s="93" t="n"/>
+      <c r="C25" s="64" t="n"/>
+      <c r="D25" s="89">
         <f>SUM(D5)+SUM(D7)+SUM(D9)+SUM(D11:D12)+SUM(D14:D16)+SUM(D18:D20)+SUM(D22)</f>
         <v/>
       </c>
-      <c r="E24" s="88">
+      <c r="E25" s="88">
         <f>SUM(E5)+SUM(E7)+SUM(E9)+SUM(E11:E12)+SUM(E14:E16)+SUM(E18:E20)+SUM(E22)</f>
         <v/>
       </c>
-      <c r="F24" s="97" t="n"/>
-      <c r="G24" s="97" t="n"/>
+      <c r="F25" s="97" t="n"/>
+      <c r="G25" s="97" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
chore(observability): backfill day-9+10 work-log entries
MAIN session: M1 close ceremony — 3hr, 8 files, Milestone Planning.
Appended to row 61 (All Sessions) + row 25 (Milestone Planning).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -32,10 +32,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="33">
     <font>
@@ -3839,7 +3840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="56" min="1" max="1"/>
@@ -3866,6 +3867,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="57">
       <c r="A4" s="78" t="inlineStr">
         <is>
@@ -5696,25 +5698,61 @@
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="106" t="inlineStr">
+    <row r="61" ht="64" customHeight="1" s="57">
+      <c r="A61" s="131" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B61" s="123" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C61" s="124" t="inlineStr">
+        <is>
+          <t>10:00 AM – 1:00 PM</t>
+        </is>
+      </c>
+      <c r="D61" s="125" t="n">
+        <v>3</v>
+      </c>
+      <c r="E61" s="123" t="n">
+        <v>8</v>
+      </c>
+      <c r="F61" s="124" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="G61" s="124" t="inlineStr">
+        <is>
+          <t>M1 close ceremony</t>
+        </is>
+      </c>
+      <c r="H61" s="124" t="inlineStr">
+        <is>
+          <t>M1 close ceremony — Day 9+10 combined. RBAC sweep 54/54 pass. Audit chain env-skip (no local DATABASE_URL). Filed m1-close-report.md (47 PRs, 358 tests, 21/41 frames, $0/month). Pushed tag m1-closed-2026-05-05. Posted m1-closed-announcement. Wrote Day-9+10-combined EOD report. PR #48 fix(web): f27 /admin/users 404 — users-api.ts relative URL fixed to NEXT_PUBLIC_API_BASE_URL (BE wiring was correct; FE bug). Bonus: better-auth pnpm hoist applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="106" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B61" s="93" t="n"/>
-      <c r="C61" s="64" t="n"/>
-      <c r="D61" s="89">
+      <c r="B62" s="93" t="n"/>
+      <c r="C62" s="64" t="n"/>
+      <c r="D62" s="89">
         <f>SUM(D5:D59)</f>
         <v/>
       </c>
-      <c r="E61" s="88">
+      <c r="E62" s="88">
         <f>SUM(E5:E59)</f>
         <v/>
       </c>
-      <c r="F61" s="97" t="n"/>
-      <c r="G61" s="97" t="n"/>
-      <c r="H61" s="97" t="n"/>
+      <c r="F62" s="97" t="n"/>
+      <c r="G62" s="97" t="n"/>
+      <c r="H62" s="97" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5734,7 +5772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P30"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5820,1710 +5858,1772 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr">
+      <c r="F2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="56" t="inlineStr"/>
+      <c r="O2" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
+      <c r="F3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="56" t="inlineStr"/>
+      <c r="O3" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="inlineStr">
+      <c r="F4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="56" t="inlineStr"/>
+      <c r="O4" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="inlineStr">
+      <c r="F5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="56" t="inlineStr"/>
+      <c r="O5" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="F6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="56" t="inlineStr"/>
+      <c r="O6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="56" t="inlineStr">
         <is>
           <t>06:00</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="56" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="56" t="n">
         <v>660</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7" s="56" t="n">
         <v>120</v>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="56" t="n">
         <v>240000</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" s="56" t="n">
         <v>60000</v>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
+      <c r="J7" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="56" t="n">
         <v>6450</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="56" t="n">
         <v>1.62</v>
       </c>
-      <c r="M7" t="n">
+      <c r="M7" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N7" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O7" t="n">
+      <c r="O7" s="56" t="n">
         <v>17</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="56" t="inlineStr">
         <is>
           <t>heuristic</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="F8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="56" t="inlineStr"/>
+      <c r="O8" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="inlineStr">
+      <c r="F9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="56" t="inlineStr"/>
+      <c r="O9" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="56" t="inlineStr">
         <is>
           <t>04:30</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="56" t="inlineStr">
         <is>
           <t>06:40</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="56" t="n">
         <v>130</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10" s="56" t="n">
         <v>85</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="56" t="n">
         <v>170000</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="56" t="n">
         <v>42500</v>
       </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
+      <c r="J10" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="56" t="n">
         <v>57400</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="56" t="n">
         <v>1.1475</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M10" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="N10" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O10" t="n">
+      <c r="O10" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="P10" s="56" t="inlineStr">
         <is>
           <t>heuristic</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="56" t="inlineStr">
         <is>
           <t>08:20</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="56" t="inlineStr">
         <is>
           <t>09:35</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="56" t="n">
         <v>75</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11" s="56" t="n">
         <v>53</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="56" t="n">
         <v>106000</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="56" t="n">
         <v>26500</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
+      <c r="J11" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="56" t="n">
         <v>18850</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="56" t="n">
         <v>0.7155</v>
       </c>
-      <c r="M11" t="n">
+      <c r="M11" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="N11" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O11" t="n">
+      <c r="O11" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" s="56" t="inlineStr">
         <is>
           <t>heuristic</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="56" t="inlineStr">
         <is>
           <t>13:35</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="56" t="inlineStr">
         <is>
           <t>15:30</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="56" t="n">
         <v>115</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12" s="56" t="n">
         <v>75</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="56" t="n">
         <v>150000</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="56" t="n">
         <v>37500</v>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
+      <c r="J12" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="56" t="n">
         <v>26800</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="56" t="n">
         <v>1.0125</v>
       </c>
-      <c r="M12" t="n">
+      <c r="M12" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N12" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O12" t="n">
+      <c r="O12" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P12" s="56" t="inlineStr">
         <is>
           <t>heuristic</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="inlineStr">
+      <c r="F13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="56" t="inlineStr"/>
+      <c r="O13" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="inlineStr">
+      <c r="F14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="56" t="inlineStr"/>
+      <c r="O14" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="inlineStr">
+      <c r="F15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="56" t="inlineStr"/>
+      <c r="O15" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="inlineStr">
+      <c r="F16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="56" t="inlineStr"/>
+      <c r="O16" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" t="inlineStr">
+      <c r="F17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="56" t="inlineStr"/>
+      <c r="O17" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="56" t="n">
         <v>4</v>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" t="inlineStr">
+      <c r="F18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="56" t="inlineStr"/>
+      <c r="O18" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="inlineStr">
+      <c r="F19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="56" t="inlineStr"/>
+      <c r="O19" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" t="inlineStr">
+      <c r="F20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="56" t="inlineStr"/>
+      <c r="O20" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="56" t="n">
         <v>5</v>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="inlineStr">
+      <c r="F21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="56" t="inlineStr"/>
+      <c r="O21" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="56" t="n">
         <v>6</v>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="inlineStr">
+      <c r="F22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="56" t="inlineStr"/>
+      <c r="O22" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="56" t="n">
         <v>6</v>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" t="inlineStr">
+      <c r="F23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="56" t="inlineStr"/>
+      <c r="O23" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="56" t="n">
         <v>6</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" t="inlineStr">
+      <c r="F24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="56" t="inlineStr"/>
+      <c r="O24" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="56" t="n">
         <v>7</v>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="n">
-        <v>0</v>
-      </c>
-      <c r="P25" t="inlineStr">
+      <c r="F25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="56" t="inlineStr"/>
+      <c r="O25" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="56" t="n">
         <v>7</v>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" t="inlineStr">
+      <c r="F26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="56" t="inlineStr"/>
+      <c r="O26" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="56" t="n">
         <v>7</v>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" t="inlineStr">
+      <c r="F27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="56" t="inlineStr"/>
+      <c r="O27" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="56" t="inlineStr">
         <is>
           <t>&lt;unknown&gt;</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="56" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>08:03</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>09:03</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
+      <c r="D28" s="56" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="E28" s="56" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="F28" s="56" t="n">
         <v>60</v>
       </c>
-      <c r="G28" t="n">
-        <v>380</v>
-      </c>
-      <c r="H28" t="n">
-        <v>14795684</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1633766</v>
-      </c>
-      <c r="J28" t="n">
-        <v>915046942</v>
-      </c>
-      <c r="K28" t="n">
-        <v>138200</v>
-      </c>
-      <c r="L28" t="n">
-        <v>354.5024</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" t="inlineStr">
+      <c r="G28" s="56" t="n">
+        <v>605</v>
+      </c>
+      <c r="H28" s="56" t="n">
+        <v>57919271</v>
+      </c>
+      <c r="I28" s="56" t="n">
+        <v>5050863</v>
+      </c>
+      <c r="J28" s="56" t="n">
+        <v>2050437403</v>
+      </c>
+      <c r="K28" s="56" t="n">
+        <v>220050</v>
+      </c>
+      <c r="L28" s="56" t="n">
+        <v>908.0778</v>
+      </c>
+      <c r="M28" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O28" t="n">
-        <v>7</v>
-      </c>
-      <c r="P28" t="inlineStr">
+      <c r="O28" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="P28" s="56" t="inlineStr">
         <is>
           <t>conversation</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="56" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>08:09</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>09:09</t>
-        </is>
-      </c>
-      <c r="F29" t="n">
+      <c r="D29" s="56" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="E29" s="56" t="inlineStr">
+        <is>
+          <t>12:44</t>
+        </is>
+      </c>
+      <c r="F29" s="56" t="n">
         <v>60</v>
       </c>
-      <c r="G29" t="n">
-        <v>395</v>
-      </c>
-      <c r="H29" t="n">
-        <v>47506810</v>
-      </c>
-      <c r="I29" t="n">
-        <v>4976422</v>
-      </c>
-      <c r="J29" t="n">
-        <v>1991637006</v>
-      </c>
-      <c r="K29" t="n">
-        <v>143550</v>
-      </c>
-      <c r="L29" t="n">
-        <v>850.2745</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" t="inlineStr">
+      <c r="G29" s="56" t="n">
+        <v>646</v>
+      </c>
+      <c r="H29" s="56" t="n">
+        <v>16906939</v>
+      </c>
+      <c r="I29" s="56" t="n">
+        <v>2050459</v>
+      </c>
+      <c r="J29" s="56" t="n">
+        <v>1102221244</v>
+      </c>
+      <c r="K29" s="56" t="n">
+        <v>235100</v>
+      </c>
+      <c r="L29" s="56" t="n">
+        <v>424.8218</v>
+      </c>
+      <c r="M29" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="56" t="inlineStr">
         <is>
           <t>main</t>
         </is>
       </c>
-      <c r="O29" t="n">
+      <c r="O29" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="P29" s="56" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="56" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="P29" t="inlineStr">
+      <c r="C30" s="56" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D30" s="56" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="E30" s="56" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="F30" s="56" t="n">
+        <v>60</v>
+      </c>
+      <c r="G30" s="56" t="n">
+        <v>656</v>
+      </c>
+      <c r="H30" s="56" t="n">
+        <v>29354349</v>
+      </c>
+      <c r="I30" s="56" t="n">
+        <v>2836353</v>
+      </c>
+      <c r="J30" s="56" t="n">
+        <v>1049822514</v>
+      </c>
+      <c r="K30" s="56" t="n">
+        <v>238400</v>
+      </c>
+      <c r="L30" s="56" t="n">
+        <v>467.5679</v>
+      </c>
+      <c r="M30" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="56" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O30" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="P30" s="56" t="inlineStr">
         <is>
           <t>conversation</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>8</v>
-      </c>
-      <c r="C30" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="56" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B31" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="C31" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>08:28</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>09:28</t>
-        </is>
-      </c>
-      <c r="F30" t="n">
-        <v>60</v>
-      </c>
-      <c r="G30" t="n">
-        <v>440</v>
-      </c>
-      <c r="H30" t="n">
-        <v>20438300</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2544848</v>
-      </c>
-      <c r="J30" t="n">
-        <v>880081747</v>
-      </c>
-      <c r="K30" t="n">
-        <v>159600</v>
-      </c>
-      <c r="L30" t="n">
-        <v>378.8384</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>chore/work-log-consolidation</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
-        <v>9</v>
-      </c>
-      <c r="P30" t="inlineStr">
+      <c r="D31" s="56" t="inlineStr">
+        <is>
+          <t>04:54</t>
+        </is>
+      </c>
+      <c r="E31" s="56" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="F31" s="56" t="n">
+        <v>483</v>
+      </c>
+      <c r="G31" s="56" t="n">
+        <v>565</v>
+      </c>
+      <c r="H31" s="56" t="n">
+        <v>1611343</v>
+      </c>
+      <c r="I31" s="56" t="n">
+        <v>253592</v>
+      </c>
+      <c r="J31" s="56" t="n">
+        <v>39486361</v>
+      </c>
+      <c r="K31" s="56" t="n">
+        <v>205250</v>
+      </c>
+      <c r="L31" s="56" t="n">
+        <v>21.6919</v>
+      </c>
+      <c r="M31" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="56" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O31" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="P31" s="56" t="inlineStr">
         <is>
           <t>conversation</t>
         </is>
@@ -7540,7 +7640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7591,96 +7691,127 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="56" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="56" t="n">
         <v>11</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="56" t="n">
         <v>120</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="56" t="n">
         <v>240000</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="56" t="n">
         <v>60000</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="56" t="n">
         <v>6450</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="56" t="n">
         <v>1.62</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="56" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="56" t="n">
         <v>5.33</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="56" t="n">
         <v>213</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="56" t="n">
         <v>426000</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="56" t="n">
         <v>106500</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="56" t="n">
         <v>103050</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="56" t="n">
         <v>2.8755</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="56" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="56" t="n">
         <v>8</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="56" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
-        <v>1215</v>
-      </c>
-      <c r="F4" t="n">
-        <v>82740794</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9155036</v>
-      </c>
-      <c r="H4" t="n">
-        <v>441350</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1583.6153</v>
+      <c r="E4" s="56" t="n">
+        <v>1907</v>
+      </c>
+      <c r="F4" s="56" t="n">
+        <v>104180559</v>
+      </c>
+      <c r="G4" s="56" t="n">
+        <v>9937675</v>
+      </c>
+      <c r="H4" s="56" t="n">
+        <v>693550</v>
+      </c>
+      <c r="I4" s="56" t="n">
+        <v>1800.4675</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="56" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="B5" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="56" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="56" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="E5" s="56" t="n">
+        <v>565</v>
+      </c>
+      <c r="F5" s="56" t="n">
+        <v>1611343</v>
+      </c>
+      <c r="G5" s="56" t="n">
+        <v>253592</v>
+      </c>
+      <c r="H5" s="56" t="n">
+        <v>205250</v>
+      </c>
+      <c r="I5" s="56" t="n">
+        <v>21.6919</v>
       </c>
     </row>
   </sheetData>
@@ -7750,71 +7881,71 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C2" t="n">
-        <v>19.33</v>
-      </c>
-      <c r="D2" t="n">
-        <v>1548</v>
-      </c>
-      <c r="E2" t="n">
-        <v>83406794</v>
-      </c>
-      <c r="F2" t="n">
-        <v>9321536</v>
-      </c>
-      <c r="G2" t="n">
-        <v>550850</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1588.1108</v>
-      </c>
-      <c r="I2" t="n">
-        <v>28497</v>
-      </c>
-      <c r="J2" t="n">
-        <v>8.949999999999999</v>
+      <c r="B2" s="56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="56" t="n">
+        <v>27.38</v>
+      </c>
+      <c r="D2" s="56" t="n">
+        <v>2805</v>
+      </c>
+      <c r="E2" s="56" t="n">
+        <v>106457902</v>
+      </c>
+      <c r="F2" s="56" t="n">
+        <v>10357767</v>
+      </c>
+      <c r="G2" s="56" t="n">
+        <v>1008300</v>
+      </c>
+      <c r="H2" s="56" t="n">
+        <v>1826.6549</v>
+      </c>
+      <c r="I2" s="56" t="n">
+        <v>36826</v>
+      </c>
+      <c r="J2" s="56" t="n">
+        <v>10.28</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>7</v>
-      </c>
-      <c r="C3" t="n">
-        <v>19.33</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1548</v>
-      </c>
-      <c r="E3" t="n">
-        <v>83406794</v>
-      </c>
-      <c r="F3" t="n">
-        <v>9321536</v>
-      </c>
-      <c r="G3" t="n">
-        <v>550850</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1588.1108</v>
-      </c>
-      <c r="I3" t="n">
-        <v>28497</v>
-      </c>
-      <c r="J3" t="n">
-        <v>8.949999999999999</v>
+      <c r="B3" s="56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="56" t="n">
+        <v>27.38</v>
+      </c>
+      <c r="D3" s="56" t="n">
+        <v>2805</v>
+      </c>
+      <c r="E3" s="56" t="n">
+        <v>106457902</v>
+      </c>
+      <c r="F3" s="56" t="n">
+        <v>10357767</v>
+      </c>
+      <c r="G3" s="56" t="n">
+        <v>1008300</v>
+      </c>
+      <c r="H3" s="56" t="n">
+        <v>1826.6549</v>
+      </c>
+      <c r="I3" s="56" t="n">
+        <v>36826</v>
+      </c>
+      <c r="J3" s="56" t="n">
+        <v>10.28</v>
       </c>
     </row>
   </sheetData>
@@ -7859,702 +7990,702 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="56" t="inlineStr">
         <is>
           <t>Tokens In/Out</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="56" t="inlineStr">
         <is>
           <t>Conversation file ~/.claude/projects/.../d1-main.jsonl missing or empty</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="56" t="inlineStr">
         <is>
           <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="56" t="inlineStr">
         <is>
           <t>Tokens In/Out</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="56" t="inlineStr">
         <is>
           <t>Conversation file ~/.claude/projects/.../d2-morni.jsonl missing or empty</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="56" t="inlineStr">
         <is>
           <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="56" t="inlineStr">
         <is>
           <t>Tokens In/Out</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="56" t="inlineStr">
         <is>
           <t>Conversation file ~/.claude/projects/.../d2-eveni.jsonl missing or empty</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="56" t="inlineStr">
         <is>
           <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="56" t="inlineStr">
         <is>
           <t>Tokens In/Out</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="56" t="inlineStr">
         <is>
           <t>Conversation file ~/.claude/projects/.../d2-stret.jsonl missing or empty</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="56" t="inlineStr">
         <is>
           <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-26 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-04-26-day-0.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="56" t="inlineStr">
         <is>
           <t>2026-04-26</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="56" t="inlineStr">
         <is>
           <t>2026-04-27</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="56" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-29 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-04-29-day-3.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="56" t="inlineStr">
         <is>
           <t>2026-04-29</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-30 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-04-30-day-4.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="56" t="inlineStr">
         <is>
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-01 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-05-01-day-5.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="56" t="inlineStr">
         <is>
           <t>2026-05-01</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-02 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-05-02-day-6.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>2026-05-02</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="56" t="inlineStr">
         <is>
           <t>MAIN</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="56" t="inlineStr">
         <is>
           <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-03 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="56" t="inlineStr">
         <is>
           <t>Reconstruct hours from docs/eod-reports/2026-05-03-day-7.md; tokens unrecoverable for past sessions</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="56" t="inlineStr">
         <is>
           <t>FE</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="56" t="inlineStr">
         <is>
           <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="56" t="inlineStr">
         <is>
           <t>2026-05-03</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="56" t="inlineStr">
         <is>
           <t>BE</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="56" t="inlineStr">
         <is>
           <t>All token + hours fields</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="56" t="inlineStr">
         <is>
           <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="56" t="inlineStr">
         <is>
           <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
         </is>
@@ -11034,7 +11165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="56" min="1" max="1"/>
@@ -11059,6 +11190,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="57">
       <c r="A4" s="78" t="inlineStr">
         <is>
@@ -11576,24 +11708,55 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="106" t="inlineStr">
+    <row r="25" ht="64" customHeight="1" s="57">
+      <c r="A25" s="131" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B25" s="123" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="C25" s="124" t="inlineStr">
+        <is>
+          <t>10:00 AM – 1:00 PM</t>
+        </is>
+      </c>
+      <c r="D25" s="125" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="123" t="n">
+        <v>8</v>
+      </c>
+      <c r="F25" s="124" t="inlineStr">
+        <is>
+          <t>M1 close ceremony</t>
+        </is>
+      </c>
+      <c r="G25" s="124" t="inlineStr">
+        <is>
+          <t>M1 close ceremony — Day 9+10 combined. RBAC sweep 54/54 pass. Audit chain env-skip (no local DATABASE_URL). Filed m1-close-report.md (47 PRs, 358 tests, 21/41 frames, $0/month). Pushed tag m1-closed-2026-05-05. Posted m1-closed-announcement. Wrote Day-9+10-combined EOD report. PR #48 fix(web): f27 /admin/users 404 — users-api.ts relative URL fixed to NEXT_PUBLIC_API_BASE_URL (BE wiring was correct; FE bug). Bonus: better-auth pnpm hoist applied.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="106" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B25" s="93" t="n"/>
-      <c r="C25" s="64" t="n"/>
-      <c r="D25" s="89">
+      <c r="B26" s="93" t="n"/>
+      <c r="C26" s="64" t="n"/>
+      <c r="D26" s="89">
         <f>SUM(D5)+SUM(D7)+SUM(D9)+SUM(D11:D12)+SUM(D14:D16)+SUM(D18:D20)+SUM(D22)</f>
         <v/>
       </c>
-      <c r="E25" s="88">
+      <c r="E26" s="88">
         <f>SUM(E5)+SUM(E7)+SUM(E9)+SUM(E11:E12)+SUM(E14:E16)+SUM(E18:E20)+SUM(E22)</f>
         <v/>
       </c>
-      <c r="F25" s="97" t="n"/>
-      <c r="G25" s="97" t="n"/>
+      <c r="F26" s="97" t="n"/>
+      <c r="G26" s="97" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>

<commit_message>
chore(observability): backfill day-11 work-log entries (3 worktrees + main sessions-stream entry)
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -31,11 +31,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -310,6 +311,10 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="44">
     <fill>
@@ -571,7 +576,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -686,6 +691,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -824,7 +843,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1087,6 +1106,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4261,7 +4292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H20"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4730,24 +4761,55 @@
       </c>
       <c r="H19" s="7" t="n"/>
     </row>
-    <row r="20" ht="24" customHeight="1" s="15">
-      <c r="B20" s="37" t="inlineStr">
+    <row r="20" ht="64" customHeight="1" s="15">
+      <c r="B20" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C20" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D20" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 4:39 PM</t>
+        </is>
+      </c>
+      <c r="E20" s="103" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F20" s="101" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="102" t="inlineStr">
+        <is>
+          <t>Day-11 M2 cascade + xlsx swap + Rule 14</t>
+        </is>
+      </c>
+      <c r="H20" s="102" t="inlineStr">
+        <is>
+          <t>MAIN session: skill audit PR #50, ctx-discipline #54, compound-learnings backfill #56, professional xlsx swap with 26-row backfill #59, Hard Rule 14 codified #64, EOD MAIN section #65. Cascade through 75min GHA outage 13:30-14:45 IST. 13+ PRs auto-merged across MAIN/BE+1/FE+1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="13">
-        <f>SUM(E6:E19)</f>
+      <c r="C21" s="54" t="n"/>
+      <c r="D21" s="54" t="n"/>
+      <c r="E21" s="13">
+        <f>SUM(E6:E20)</f>
         <v/>
       </c>
-      <c r="F20" s="14">
-        <f>SUM(F6:F19)</f>
+      <c r="F21" s="14">
+        <f>SUM(F6:F20)</f>
         <v/>
       </c>
-      <c r="G20" s="54" t="n"/>
-      <c r="H20" s="54" t="n"/>
+      <c r="G21" s="54" t="n"/>
+      <c r="H21" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4892,7 +4954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4904,6 +4966,7 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4918,6 +4981,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5299,24 +5363,86 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="37" t="inlineStr">
+    <row r="18" ht="64" customHeight="1" s="15">
+      <c r="B18" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C18" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D18" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 5:45 PM</t>
+        </is>
+      </c>
+      <c r="E18" s="103" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F18" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="102" t="inlineStr">
+        <is>
+          <t>M2 TASK 1 F12 KB Upload + AdminShell fix</t>
+        </is>
+      </c>
+      <c r="H18" s="102" t="inlineStr">
+        <is>
+          <t>FE+1 session: F12 KB Upload Modal Pattern A scaffold (PR #52, merged 12:13 IST), AdminShell wrap fix on F12+F13 (PR #63, post visual-gate catch), Day-11 EOD + compound-learnings + sessions-stream init (PR #55). Idle Thu morning until BE /api/kb/upload-init lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="64" customHeight="1" s="15">
+      <c r="B19" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C19" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D19" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 3:30 PM</t>
+        </is>
+      </c>
+      <c r="E19" s="103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="101" t="n">
+        <v>25</v>
+      </c>
+      <c r="G19" s="102" t="inlineStr">
+        <is>
+          <t>M2 deploy + chunk-search + RAG pipeline</t>
+        </is>
+      </c>
+      <c r="H19" s="102" t="inlineStr">
+        <is>
+          <t>BE+1 session: M2 staging deploy artifacts + ADR-011 (PR #51 rebased to 577e975), chunk-search real pgvector flip (PR #53), KB RAG /api/kb/answer + ADR-012 (PR #57). 14 new tests, 325/325 BE suite. Compound-learning: citation marker = chunk header (no drift).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C18" s="54" t="n"/>
-      <c r="D18" s="54" t="n"/>
-      <c r="E18" s="13">
-        <f>SUM(E6:E17)</f>
+      <c r="C20" s="54" t="n"/>
+      <c r="D20" s="54" t="n"/>
+      <c r="E20" s="13">
+        <f>SUM(E6:E19)</f>
         <v/>
       </c>
-      <c r="F18" s="14">
-        <f>SUM(F6:F17)</f>
+      <c r="F20" s="14">
+        <f>SUM(F6:F19)</f>
         <v/>
       </c>
-      <c r="G18" s="54" t="n"/>
-      <c r="H18" s="54" t="n"/>
+      <c r="G20" s="54" t="n"/>
+      <c r="H20" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5548,7 +5674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J63"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5563,6 +5689,7 @@
     <col width="50" customWidth="1" style="15" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -5577,6 +5704,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -7562,25 +7690,136 @@
       </c>
       <c r="I62" s="5" t="n"/>
     </row>
-    <row r="63" ht="24" customHeight="1" s="15">
-      <c r="B63" s="37" t="inlineStr">
+    <row r="63" ht="64" customHeight="1" s="15">
+      <c r="B63" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C63" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D63" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 4:39 PM</t>
+        </is>
+      </c>
+      <c r="E63" s="103" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F63" s="101" t="n">
+        <v>30</v>
+      </c>
+      <c r="G63" s="102" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="H63" s="102" t="inlineStr">
+        <is>
+          <t>Day-11 M2 cascade + xlsx swap + Rule 14</t>
+        </is>
+      </c>
+      <c r="I63" s="102" t="inlineStr">
+        <is>
+          <t>MAIN session: skill audit PR #50, ctx-discipline #54, compound-learnings backfill #56, professional xlsx swap with 26-row backfill #59, Hard Rule 14 codified #64, EOD MAIN section #65. Cascade through 75min GHA outage 13:30-14:45 IST. 13+ PRs auto-merged across MAIN/BE+1/FE+1.</t>
+        </is>
+      </c>
+      <c r="J63" s="102" t="n"/>
+    </row>
+    <row r="64" ht="64" customHeight="1" s="15">
+      <c r="B64" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C64" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D64" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 5:45 PM</t>
+        </is>
+      </c>
+      <c r="E64" s="103" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F64" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G64" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H64" s="102" t="inlineStr">
+        <is>
+          <t>M2 TASK 1 F12 KB Upload + AdminShell fix</t>
+        </is>
+      </c>
+      <c r="I64" s="102" t="inlineStr">
+        <is>
+          <t>FE+1 session: F12 KB Upload Modal Pattern A scaffold (PR #52, merged 12:13 IST), AdminShell wrap fix on F12+F13 (PR #63, post visual-gate catch), Day-11 EOD + compound-learnings + sessions-stream init (PR #55). Idle Thu morning until BE /api/kb/upload-init lands.</t>
+        </is>
+      </c>
+      <c r="J64" s="102" t="n"/>
+    </row>
+    <row r="65" ht="64" customHeight="1" s="15">
+      <c r="B65" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C65" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D65" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 3:30 PM</t>
+        </is>
+      </c>
+      <c r="E65" s="103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="101" t="n">
+        <v>25</v>
+      </c>
+      <c r="G65" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H65" s="102" t="inlineStr">
+        <is>
+          <t>M2 deploy + chunk-search + RAG pipeline</t>
+        </is>
+      </c>
+      <c r="I65" s="102" t="inlineStr">
+        <is>
+          <t>BE+1 session: M2 staging deploy artifacts + ADR-011 (PR #51 rebased to 577e975), chunk-search real pgvector flip (PR #53), KB RAG /api/kb/answer + ADR-012 (PR #57). 14 new tests, 325/325 BE suite. Compound-learning: citation marker = chunk header (no drift).</t>
+        </is>
+      </c>
+      <c r="J65" s="102" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C63" s="54" t="n"/>
-      <c r="D63" s="54" t="n"/>
-      <c r="E63" s="72">
-        <f>SUM(E6:E62)</f>
+      <c r="C66" s="54" t="n"/>
+      <c r="D66" s="54" t="n"/>
+      <c r="E66" s="72">
+        <f>SUM(E6:E65)</f>
         <v/>
       </c>
-      <c r="F63" s="14">
-        <f>SUM(F6:F62)</f>
+      <c r="F66" s="14">
+        <f>SUM(F6:F65)</f>
         <v/>
       </c>
-      <c r="G63" s="54" t="n"/>
-      <c r="H63" s="54" t="n"/>
-      <c r="I63" s="54" t="n"/>
+      <c r="G66" s="54" t="n"/>
+      <c r="H66" s="54" t="n"/>
+      <c r="I66" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore(observability): backfill day-11 work-log entries (3 worktrees + main sessions-stream entry) (#67)
Co-authored-by: Yogesh Mohite <yogeshmohite@MacBookAir.bwrouter>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -31,11 +31,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="39">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -310,6 +311,10 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="44">
     <fill>
@@ -571,7 +576,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -686,6 +691,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
@@ -824,7 +843,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1087,6 +1106,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4261,7 +4292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H20"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4730,24 +4761,55 @@
       </c>
       <c r="H19" s="7" t="n"/>
     </row>
-    <row r="20" ht="24" customHeight="1" s="15">
-      <c r="B20" s="37" t="inlineStr">
+    <row r="20" ht="64" customHeight="1" s="15">
+      <c r="B20" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C20" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D20" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 4:39 PM</t>
+        </is>
+      </c>
+      <c r="E20" s="103" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F20" s="101" t="n">
+        <v>30</v>
+      </c>
+      <c r="G20" s="102" t="inlineStr">
+        <is>
+          <t>Day-11 M2 cascade + xlsx swap + Rule 14</t>
+        </is>
+      </c>
+      <c r="H20" s="102" t="inlineStr">
+        <is>
+          <t>MAIN session: skill audit PR #50, ctx-discipline #54, compound-learnings backfill #56, professional xlsx swap with 26-row backfill #59, Hard Rule 14 codified #64, EOD MAIN section #65. Cascade through 75min GHA outage 13:30-14:45 IST. 13+ PRs auto-merged across MAIN/BE+1/FE+1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="13">
-        <f>SUM(E6:E19)</f>
+      <c r="C21" s="54" t="n"/>
+      <c r="D21" s="54" t="n"/>
+      <c r="E21" s="13">
+        <f>SUM(E6:E20)</f>
         <v/>
       </c>
-      <c r="F20" s="14">
-        <f>SUM(F6:F19)</f>
+      <c r="F21" s="14">
+        <f>SUM(F6:F20)</f>
         <v/>
       </c>
-      <c r="G20" s="54" t="n"/>
-      <c r="H20" s="54" t="n"/>
+      <c r="G21" s="54" t="n"/>
+      <c r="H21" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4892,7 +4954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H18"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4904,6 +4966,7 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4918,6 +4981,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5299,24 +5363,86 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="37" t="inlineStr">
+    <row r="18" ht="64" customHeight="1" s="15">
+      <c r="B18" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C18" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D18" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 5:45 PM</t>
+        </is>
+      </c>
+      <c r="E18" s="103" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F18" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G18" s="102" t="inlineStr">
+        <is>
+          <t>M2 TASK 1 F12 KB Upload + AdminShell fix</t>
+        </is>
+      </c>
+      <c r="H18" s="102" t="inlineStr">
+        <is>
+          <t>FE+1 session: F12 KB Upload Modal Pattern A scaffold (PR #52, merged 12:13 IST), AdminShell wrap fix on F12+F13 (PR #63, post visual-gate catch), Day-11 EOD + compound-learnings + sessions-stream init (PR #55). Idle Thu morning until BE /api/kb/upload-init lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="64" customHeight="1" s="15">
+      <c r="B19" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C19" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D19" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 3:30 PM</t>
+        </is>
+      </c>
+      <c r="E19" s="103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F19" s="101" t="n">
+        <v>25</v>
+      </c>
+      <c r="G19" s="102" t="inlineStr">
+        <is>
+          <t>M2 deploy + chunk-search + RAG pipeline</t>
+        </is>
+      </c>
+      <c r="H19" s="102" t="inlineStr">
+        <is>
+          <t>BE+1 session: M2 staging deploy artifacts + ADR-011 (PR #51 rebased to 577e975), chunk-search real pgvector flip (PR #53), KB RAG /api/kb/answer + ADR-012 (PR #57). 14 new tests, 325/325 BE suite. Compound-learning: citation marker = chunk header (no drift).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C18" s="54" t="n"/>
-      <c r="D18" s="54" t="n"/>
-      <c r="E18" s="13">
-        <f>SUM(E6:E17)</f>
+      <c r="C20" s="54" t="n"/>
+      <c r="D20" s="54" t="n"/>
+      <c r="E20" s="13">
+        <f>SUM(E6:E19)</f>
         <v/>
       </c>
-      <c r="F18" s="14">
-        <f>SUM(F6:F17)</f>
+      <c r="F20" s="14">
+        <f>SUM(F6:F19)</f>
         <v/>
       </c>
-      <c r="G18" s="54" t="n"/>
-      <c r="H18" s="54" t="n"/>
+      <c r="G20" s="54" t="n"/>
+      <c r="H20" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5548,7 +5674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J63"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5563,6 +5689,7 @@
     <col width="50" customWidth="1" style="15" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -5577,6 +5704,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -7562,25 +7690,136 @@
       </c>
       <c r="I62" s="5" t="n"/>
     </row>
-    <row r="63" ht="24" customHeight="1" s="15">
-      <c r="B63" s="37" t="inlineStr">
+    <row r="63" ht="64" customHeight="1" s="15">
+      <c r="B63" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C63" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D63" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 4:39 PM</t>
+        </is>
+      </c>
+      <c r="E63" s="103" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F63" s="101" t="n">
+        <v>30</v>
+      </c>
+      <c r="G63" s="102" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="H63" s="102" t="inlineStr">
+        <is>
+          <t>Day-11 M2 cascade + xlsx swap + Rule 14</t>
+        </is>
+      </c>
+      <c r="I63" s="102" t="inlineStr">
+        <is>
+          <t>MAIN session: skill audit PR #50, ctx-discipline #54, compound-learnings backfill #56, professional xlsx swap with 26-row backfill #59, Hard Rule 14 codified #64, EOD MAIN section #65. Cascade through 75min GHA outage 13:30-14:45 IST. 13+ PRs auto-merged across MAIN/BE+1/FE+1.</t>
+        </is>
+      </c>
+      <c r="J63" s="102" t="n"/>
+    </row>
+    <row r="64" ht="64" customHeight="1" s="15">
+      <c r="B64" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C64" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D64" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 5:45 PM</t>
+        </is>
+      </c>
+      <c r="E64" s="103" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F64" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G64" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H64" s="102" t="inlineStr">
+        <is>
+          <t>M2 TASK 1 F12 KB Upload + AdminShell fix</t>
+        </is>
+      </c>
+      <c r="I64" s="102" t="inlineStr">
+        <is>
+          <t>FE+1 session: F12 KB Upload Modal Pattern A scaffold (PR #52, merged 12:13 IST), AdminShell wrap fix on F12+F13 (PR #63, post visual-gate catch), Day-11 EOD + compound-learnings + sessions-stream init (PR #55). Idle Thu morning until BE /api/kb/upload-init lands.</t>
+        </is>
+      </c>
+      <c r="J64" s="102" t="n"/>
+    </row>
+    <row r="65" ht="64" customHeight="1" s="15">
+      <c r="B65" s="100" t="n">
+        <v>46148</v>
+      </c>
+      <c r="C65" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D65" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 3:30 PM</t>
+        </is>
+      </c>
+      <c r="E65" s="103" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" s="101" t="n">
+        <v>25</v>
+      </c>
+      <c r="G65" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H65" s="102" t="inlineStr">
+        <is>
+          <t>M2 deploy + chunk-search + RAG pipeline</t>
+        </is>
+      </c>
+      <c r="I65" s="102" t="inlineStr">
+        <is>
+          <t>BE+1 session: M2 staging deploy artifacts + ADR-011 (PR #51 rebased to 577e975), chunk-search real pgvector flip (PR #53), KB RAG /api/kb/answer + ADR-012 (PR #57). 14 new tests, 325/325 BE suite. Compound-learning: citation marker = chunk header (no drift).</t>
+        </is>
+      </c>
+      <c r="J65" s="102" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C63" s="54" t="n"/>
-      <c r="D63" s="54" t="n"/>
-      <c r="E63" s="72">
-        <f>SUM(E6:E62)</f>
+      <c r="C66" s="54" t="n"/>
+      <c r="D66" s="54" t="n"/>
+      <c r="E66" s="72">
+        <f>SUM(E6:E65)</f>
         <v/>
       </c>
-      <c r="F63" s="14">
-        <f>SUM(F6:F62)</f>
+      <c r="F66" s="14">
+        <f>SUM(F6:F65)</f>
         <v/>
       </c>
-      <c r="G63" s="54" t="n"/>
-      <c r="H63" s="54" t="n"/>
-      <c r="I63" s="54" t="n"/>
+      <c r="G66" s="54" t="n"/>
+      <c r="H66" s="54" t="n"/>
+      <c r="I66" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore(observability): backfill day-12 work-log entries
Add MAIN session row for 2026-05-07 to All Sessions sheet:
06:50-17:00 IST, 10.2 hr, 18 files, "Milestone Planning" phase,
theme "Day-12 / M2 Close Ceremony — 2-day vs 4-day plan".

Description covers: morning audits + observability (#67/#68/#76),
M2 critical-path cascade (#69/#71/#72/#78/#79/#80), close ceremony
steps 1-8 (#81 close report, #82 EOD, tag m2-closed-2026-05-07).

Token sessions for 2026-05-07 — source rebuild ran but didn't pick
up today's entries (script reads pre-computed data); same gap as
day-11. Carry to fri am for proper backfill.

Sessions-stream auto-appended by stop hook (3 main entries).
Fe+1 + be+1 entries will append when their stop hooks fire.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -13,16 +13,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Sessions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Daily Rollup" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Token Comparison" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backfill_Notes" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Report" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Idea Confirmation" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Management Research" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Automation &amp; Reporting" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design &amp; Specifications" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Planning" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Creative" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consolidated Report" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Idea Confirmation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Case Management Research" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Automation &amp; Reporting" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design &amp; Specifications" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestone Planning" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Launch Creative" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Development" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tokens — Sessions" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tokens — Daily Rollup" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tokens — Per-Chat Comparison" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backfill_Notes" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -36,7 +39,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="41">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -315,8 +318,12 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="44">
+  <fills count="45">
     <fill>
       <patternFill/>
     </fill>
@@ -573,6 +580,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F766E"/>
+        <bgColor rgb="000F766E"/>
       </patternFill>
     </fill>
   </fills>
@@ -843,7 +856,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1117,6 +1130,9 @@
     </xf>
     <xf numFmtId="2" fontId="39" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3059,162 +3075,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8" outlineLevelRow="7"/>
-  <cols>
-    <col width="3" customWidth="1" style="15" min="1" max="1"/>
-    <col width="14" customWidth="1" style="15" min="2" max="2"/>
-    <col width="12" customWidth="1" style="15" min="3" max="3"/>
-    <col width="22" customWidth="1" style="15" min="4" max="4"/>
-    <col width="12" customWidth="1" style="15" min="5" max="6"/>
-    <col width="42" customWidth="1" style="15" min="7" max="7"/>
-    <col width="50" customWidth="1" style="15" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="31.5" customHeight="1" s="15">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Idea Confirmation — Session Evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="27.75" customHeight="1" s="15">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Phase 1 — vision, market research, problem statement, solution design, mockups, competitive analysis, flow diagrams.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" s="15">
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Timing</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Hours</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Files</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Evidence / Theme</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>What I Did</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="19.5" customHeight="1" s="15">
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>10:28 PM – 10:28 PM</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>QA_Nexus_Brainstorm.md</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="19.5" customHeight="1" s="15">
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>2026-04-17</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>8:22 PM – 11:30 PM</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>3.37</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>QA_Roles_Documents_Reference_Guide.md · QA_Nexus_Platform_Vision.md · problem-landscape.drawio</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="24" customHeight="1" s="15">
-      <c r="B8" s="37" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="C8" s="54" t="n"/>
-      <c r="D8" s="54" t="n"/>
-      <c r="E8" s="13">
-        <f>SUM(E6:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="14">
-        <f>SUM(F6:F7)</f>
-        <v/>
-      </c>
-      <c r="G8" s="54" t="n"/>
-      <c r="H8" s="54" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B2:H2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="B2:H9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
@@ -3394,7 +3254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3550,7 +3410,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4286,13 +4146,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H21"/>
+  <dimension ref="B2:H22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4792,24 +4652,55 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="37" t="inlineStr">
+    <row r="21" ht="64" customHeight="1" s="15">
+      <c r="B21" s="100" t="n">
+        <v>46149</v>
+      </c>
+      <c r="C21" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D21" s="102" t="inlineStr">
+        <is>
+          <t>06:50 AM – 5:00 PM</t>
+        </is>
+      </c>
+      <c r="E21" s="103" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F21" s="101" t="n">
+        <v>18</v>
+      </c>
+      <c r="G21" s="102" t="inlineStr">
+        <is>
+          <t>Day-12 / M2 Close Ceremony — 2-day vs 4-day plan</t>
+        </is>
+      </c>
+      <c r="H21" s="102" t="inlineStr">
+        <is>
+          <t>M2 closed 2 days ahead of plan (2x cadence). 16 PRs merged today across MAIN orchestration: morning Hard Rule 14 retrofit audit (#68), sessions-stream correlation hook (#76), Day-11 backfill (#67); afternoon BE/FE M2 cascade: prettier-write fix (#79) unblocking #77 #78; #78 BE M2 KB doc-create endpoint closes (al) blocker; #69 AdminShell v2 + #71 F13 flip + #80 F12 flip + #72 F15 flip merged in 16-min burst at 15:36-15:52 IST once visual-gate flags dropped; ceremony at 16:00-16:38 IST: close-gate sweep 69/69 ✅, audit chain env-skip documented, close report drafted (#81), tag m2-closed-2026-05-07 pushed at commit 498f206, EOD report drafted (#82). Carry-overs: (am) Rule 14 retrofit on F08+F09, (ae) embedding-spec direction call, Render staging Yogesh action, (ap) playwright cold-install cache.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C21" s="54" t="n"/>
-      <c r="D21" s="54" t="n"/>
-      <c r="E21" s="13">
-        <f>SUM(E6:E20)</f>
+      <c r="C22" s="54" t="n"/>
+      <c r="D22" s="54" t="n"/>
+      <c r="E22" s="13">
+        <f>SUM(E6:E21)</f>
         <v/>
       </c>
-      <c r="F21" s="14">
-        <f>SUM(F6:F20)</f>
+      <c r="F22" s="14">
+        <f>SUM(F6:F21)</f>
         <v/>
       </c>
-      <c r="G21" s="54" t="n"/>
-      <c r="H21" s="54" t="n"/>
+      <c r="G22" s="54" t="n"/>
+      <c r="H22" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4821,7 +4712,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4948,13 +4839,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="B2:H20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4966,7 +4857,6 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4981,7 +4871,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5454,7 +5343,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5668,13 +5557,2200 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="104" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="inlineStr">
+        <is>
+          <t>Day-N</t>
+        </is>
+      </c>
+      <c r="C1" s="104" t="inlineStr">
+        <is>
+          <t>Worktree</t>
+        </is>
+      </c>
+      <c r="D1" s="104" t="inlineStr">
+        <is>
+          <t>Started</t>
+        </is>
+      </c>
+      <c r="E1" s="104" t="inlineStr">
+        <is>
+          <t>Ended</t>
+        </is>
+      </c>
+      <c r="F1" s="104" t="inlineStr">
+        <is>
+          <t>Duration (min)</t>
+        </is>
+      </c>
+      <c r="G1" s="104" t="inlineStr">
+        <is>
+          <t>Tool Calls</t>
+        </is>
+      </c>
+      <c r="H1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens In</t>
+        </is>
+      </c>
+      <c r="I1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens Out</t>
+        </is>
+      </c>
+      <c r="J1" s="104" t="inlineStr">
+        <is>
+          <t>Cache Read</t>
+        </is>
+      </c>
+      <c r="K1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens Saved</t>
+        </is>
+      </c>
+      <c r="L1" s="104" t="inlineStr">
+        <is>
+          <t>Cost USD</t>
+        </is>
+      </c>
+      <c r="M1" s="104" t="inlineStr">
+        <is>
+          <t>In:Out Ratio</t>
+        </is>
+      </c>
+      <c r="N1" s="104" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="O1" s="104" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="P1" s="104" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>660</v>
+      </c>
+      <c r="G7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H7" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I7" t="n">
+        <v>60000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6450</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>17</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>heuristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>130</v>
+      </c>
+      <c r="G10" t="n">
+        <v>85</v>
+      </c>
+      <c r="H10" t="n">
+        <v>170000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>42500</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>57400</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.1475</v>
+      </c>
+      <c r="M10" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>5</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>heuristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>08:20</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>75</v>
+      </c>
+      <c r="G11" t="n">
+        <v>53</v>
+      </c>
+      <c r="H11" t="n">
+        <v>106000</v>
+      </c>
+      <c r="I11" t="n">
+        <v>26500</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>18850</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.7155</v>
+      </c>
+      <c r="M11" t="n">
+        <v>4</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>heuristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>13:35</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>115</v>
+      </c>
+      <c r="G12" t="n">
+        <v>75</v>
+      </c>
+      <c r="H12" t="n">
+        <v>150000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>37500</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>26800</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.0125</v>
+      </c>
+      <c r="M12" t="n">
+        <v>4</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>4</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>heuristic</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>7</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>&lt;unknown&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>60</v>
+      </c>
+      <c r="G28" t="n">
+        <v>605</v>
+      </c>
+      <c r="H28" t="n">
+        <v>57919271</v>
+      </c>
+      <c r="I28" t="n">
+        <v>5050863</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2050437403</v>
+      </c>
+      <c r="K28" t="n">
+        <v>220050</v>
+      </c>
+      <c r="L28" t="n">
+        <v>908.0778</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>12</v>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>10</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>10:06</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>11:06</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>60</v>
+      </c>
+      <c r="G29" t="n">
+        <v>654</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22571430</v>
+      </c>
+      <c r="I29" t="n">
+        <v>2637426</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1440872447</v>
+      </c>
+      <c r="K29" t="n">
+        <v>237900</v>
+      </c>
+      <c r="L29" t="n">
+        <v>556.4628</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>chore/claude-rule-14-app-shell-parity</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>15</v>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>10</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>59</v>
+      </c>
+      <c r="G30" t="n">
+        <v>670</v>
+      </c>
+      <c r="H30" t="n">
+        <v>8749961</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1167481</v>
+      </c>
+      <c r="J30" t="n">
+        <v>608246985</v>
+      </c>
+      <c r="K30" t="n">
+        <v>243500</v>
+      </c>
+      <c r="L30" t="n">
+        <v>232.7961</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>docs/eod-day-11-main-section</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>16</v>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>10</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>11:11</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>60</v>
+      </c>
+      <c r="G31" t="n">
+        <v>673</v>
+      </c>
+      <c r="H31" t="n">
+        <v>33174972</v>
+      </c>
+      <c r="I31" t="n">
+        <v>3339822</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1218131070</v>
+      </c>
+      <c r="K31" t="n">
+        <v>245050</v>
+      </c>
+      <c r="L31" t="n">
+        <v>539.9391000000001</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>docs/eod-day-11-main-section</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>16</v>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="104" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="inlineStr">
+        <is>
+          <t>Day-N</t>
+        </is>
+      </c>
+      <c r="C1" s="104" t="inlineStr">
+        <is>
+          <t>Total Sessions</t>
+        </is>
+      </c>
+      <c r="D1" s="104" t="inlineStr">
+        <is>
+          <t>Total Hours</t>
+        </is>
+      </c>
+      <c r="E1" s="104" t="inlineStr">
+        <is>
+          <t>Total Tool Calls</t>
+        </is>
+      </c>
+      <c r="F1" s="104" t="inlineStr">
+        <is>
+          <t>Total Tokens In</t>
+        </is>
+      </c>
+      <c r="G1" s="104" t="inlineStr">
+        <is>
+          <t>Total Tokens Out</t>
+        </is>
+      </c>
+      <c r="H1" s="104" t="inlineStr">
+        <is>
+          <t>Total Tokens Saved</t>
+        </is>
+      </c>
+      <c r="I1" s="104" t="inlineStr">
+        <is>
+          <t>Total Cost USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>120</v>
+      </c>
+      <c r="F2" t="n">
+        <v>240000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>60000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6450</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.62</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5.33</v>
+      </c>
+      <c r="E3" t="n">
+        <v>213</v>
+      </c>
+      <c r="F3" t="n">
+        <v>426000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>106500</v>
+      </c>
+      <c r="H3" t="n">
+        <v>103050</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.8755</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>605</v>
+      </c>
+      <c r="F4" t="n">
+        <v>57919271</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5050863</v>
+      </c>
+      <c r="H4" t="n">
+        <v>220050</v>
+      </c>
+      <c r="I4" t="n">
+        <v>908.0778</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1997</v>
+      </c>
+      <c r="F5" t="n">
+        <v>64496363</v>
+      </c>
+      <c r="G5" t="n">
+        <v>7144729</v>
+      </c>
+      <c r="H5" t="n">
+        <v>726450</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1329.198</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="104" t="inlineStr">
+        <is>
+          <t>Worktree</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="inlineStr">
+        <is>
+          <t>Sessions</t>
+        </is>
+      </c>
+      <c r="C1" s="104" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="D1" s="104" t="inlineStr">
+        <is>
+          <t>Tool Calls</t>
+        </is>
+      </c>
+      <c r="E1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens In</t>
+        </is>
+      </c>
+      <c r="F1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens Out</t>
+        </is>
+      </c>
+      <c r="G1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens Saved</t>
+        </is>
+      </c>
+      <c r="H1" s="104" t="inlineStr">
+        <is>
+          <t>Cost USD</t>
+        </is>
+      </c>
+      <c r="I1" s="104" t="inlineStr">
+        <is>
+          <t>Tokens Saved/Hour</t>
+        </is>
+      </c>
+      <c r="J1" s="104" t="inlineStr">
+        <is>
+          <t>In:Out Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>20.32</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2935</v>
+      </c>
+      <c r="E2" t="n">
+        <v>123081634</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12362092</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1056000</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2241.7713</v>
+      </c>
+      <c r="I2" t="n">
+        <v>51969</v>
+      </c>
+      <c r="J2" t="n">
+        <v>9.960000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>20.32</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2935</v>
+      </c>
+      <c r="E3" t="n">
+        <v>123081634</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12362092</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1056000</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2241.7713</v>
+      </c>
+      <c r="I3" t="n">
+        <v>51969</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9.960000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="B2:J67"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5689,7 +7765,6 @@
     <col width="50" customWidth="1" style="15" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -5704,7 +7779,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -7801,25 +9875,62 @@
       </c>
       <c r="J65" s="102" t="n"/>
     </row>
-    <row r="66">
-      <c r="B66" s="37" t="inlineStr">
+    <row r="66" ht="64" customHeight="1" s="15">
+      <c r="B66" s="100" t="n">
+        <v>46149</v>
+      </c>
+      <c r="C66" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D66" s="102" t="inlineStr">
+        <is>
+          <t>06:50 AM – 5:00 PM</t>
+        </is>
+      </c>
+      <c r="E66" s="103" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="F66" s="101" t="n">
+        <v>18</v>
+      </c>
+      <c r="G66" s="102" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="H66" s="102" t="inlineStr">
+        <is>
+          <t>Day-12 / M2 Close Ceremony — 2-day vs 4-day plan</t>
+        </is>
+      </c>
+      <c r="I66" s="102" t="inlineStr">
+        <is>
+          <t>M2 closed 2 days ahead of plan (2x cadence). 16 PRs merged today across MAIN orchestration: morning Hard Rule 14 retrofit audit (#68), sessions-stream correlation hook (#76), Day-11 backfill (#67); afternoon BE/FE M2 cascade: prettier-write fix (#79) unblocking #77 #78; #78 BE M2 KB doc-create endpoint closes (al) blocker; #69 AdminShell v2 + #71 F13 flip + #80 F12 flip + #72 F15 flip merged in 16-min burst at 15:36-15:52 IST once visual-gate flags dropped; ceremony at 16:00-16:38 IST: close-gate sweep 69/69 ✅, audit chain env-skip documented, close report drafted (#81), tag m2-closed-2026-05-07 pushed at commit 498f206, EOD report drafted (#82). Carry-overs: (am) Rule 14 retrofit on F08+F09, (ae) embedding-spec direction call, Render staging Yogesh action, (ap) playwright cold-install cache.</t>
+        </is>
+      </c>
+      <c r="J66" s="102" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C66" s="54" t="n"/>
-      <c r="D66" s="54" t="n"/>
-      <c r="E66" s="72">
-        <f>SUM(E6:E65)</f>
+      <c r="C67" s="54" t="n"/>
+      <c r="D67" s="54" t="n"/>
+      <c r="E67" s="72">
+        <f>SUM(E6:E66)</f>
         <v/>
       </c>
-      <c r="F66" s="14">
-        <f>SUM(F6:F65)</f>
+      <c r="F67" s="14">
+        <f>SUM(F6:F66)</f>
         <v/>
       </c>
-      <c r="G66" s="54" t="n"/>
-      <c r="H66" s="54" t="n"/>
-      <c r="I66" s="54" t="n"/>
+      <c r="G67" s="54" t="n"/>
+      <c r="H67" s="54" t="n"/>
+      <c r="I67" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7837,6 +9948,749 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="104" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="inlineStr">
+        <is>
+          <t>Worktree</t>
+        </is>
+      </c>
+      <c r="C1" s="104" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="D1" s="104" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="E1" s="104" t="inlineStr">
+        <is>
+          <t>Mitigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Tokens In/Out</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Conversation file ~/.claude/projects/.../d1-main.jsonl missing or empty</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Tokens In/Out</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Conversation file ~/.claude/projects/.../d2-morni.jsonl missing or empty</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tokens In/Out</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Conversation file ~/.claude/projects/.../d2-eveni.jsonl missing or empty</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Tokens In/Out</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Conversation file ~/.claude/projects/.../d2-stret.jsonl missing or empty</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-26 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-04-26-day-0.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-29 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-04-29-day-3.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-30 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-04-30-day-4.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-01 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-05-01-day-5.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-02 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-05-02-day-6.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-03 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Reconstruct hours from docs/eod-reports/2026-05-03-day-7.md; tokens unrecoverable for past sessions</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FE</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>All token + hours fields</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -11193,776 +14047,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F31"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
-  <cols>
-    <col width="3" customWidth="1" style="15" min="1" max="1"/>
-    <col width="12" customWidth="1" style="15" min="2" max="2"/>
-    <col width="10" customWidth="1" style="15" min="3" max="3"/>
-    <col width="18" customWidth="1" style="15" min="4" max="4"/>
-    <col width="55" customWidth="1" style="15" min="5" max="5"/>
-    <col width="50" customWidth="1" style="15" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="31.5" customHeight="1" s="15">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Backfill Notes — Data Quality Transparency</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="15">
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>Explicit flags for token data gaps and mitigation strategies · All estimates are conservative</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1" s="15">
-      <c r="B5" s="42" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C5" s="42" t="inlineStr">
-        <is>
-          <t>Worktree</t>
-        </is>
-      </c>
-      <c r="D5" s="42" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="E5" s="42" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
-      <c r="F5" s="42" t="inlineStr">
-        <is>
-          <t>Mitigation</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1" s="15">
-      <c r="B6" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C6" s="48" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D6" s="48" t="inlineStr">
-        <is>
-          <t>Tokens In/Out</t>
-        </is>
-      </c>
-      <c r="E6" s="48" t="inlineStr">
-        <is>
-          <t>Conversation file ~/.claude/projects/.../d1-main.jsonl missing or empty</t>
-        </is>
-      </c>
-      <c r="F6" s="48" t="inlineStr">
-        <is>
-          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1" s="15">
-      <c r="B7" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C7" s="49" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D7" s="49" t="inlineStr">
-        <is>
-          <t>Tokens In/Out</t>
-        </is>
-      </c>
-      <c r="E7" s="49" t="inlineStr">
-        <is>
-          <t>Conversation file ~/.claude/projects/.../d2-morni.jsonl missing or empty</t>
-        </is>
-      </c>
-      <c r="F7" s="49" t="inlineStr">
-        <is>
-          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1" s="15">
-      <c r="B8" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C8" s="48" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D8" s="48" t="inlineStr">
-        <is>
-          <t>Tokens In/Out</t>
-        </is>
-      </c>
-      <c r="E8" s="48" t="inlineStr">
-        <is>
-          <t>Conversation file ~/.claude/projects/.../d2-eveni.jsonl missing or empty</t>
-        </is>
-      </c>
-      <c r="F8" s="48" t="inlineStr">
-        <is>
-          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1" s="15">
-      <c r="B9" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C9" s="49" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D9" s="49" t="inlineStr">
-        <is>
-          <t>Tokens In/Out</t>
-        </is>
-      </c>
-      <c r="E9" s="49" t="inlineStr">
-        <is>
-          <t>Conversation file ~/.claude/projects/.../d2-stret.jsonl missing or empty</t>
-        </is>
-      </c>
-      <c r="F9" s="49" t="inlineStr">
-        <is>
-          <t>Heuristic estimate (tool_calls × 2000 in / × 500 out); refine when conversation reachable</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1" s="15">
-      <c r="B10" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C10" s="48" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D10" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E10" s="48" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-26 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F10" s="48" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-04-26-day-0.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1" s="15">
-      <c r="B11" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C11" s="49" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D11" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E11" s="49" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F11" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1" s="15">
-      <c r="B12" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-26</t>
-        </is>
-      </c>
-      <c r="C12" s="48" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D12" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E12" s="48" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F12" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1" s="15">
-      <c r="B13" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C13" s="49" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D13" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E13" s="49" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F13" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1" s="15">
-      <c r="B14" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-27</t>
-        </is>
-      </c>
-      <c r="C14" s="48" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D14" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E14" s="48" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F14" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1" s="15">
-      <c r="B15" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C15" s="49" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D15" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E15" s="49" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F15" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1" s="15">
-      <c r="B16" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-28</t>
-        </is>
-      </c>
-      <c r="C16" s="48" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D16" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E16" s="48" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F16" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1" s="15">
-      <c r="B17" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C17" s="49" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D17" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E17" s="49" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-29 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F17" s="49" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-04-29-day-3.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1" s="15">
-      <c r="B18" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D18" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E18" s="48" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F18" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1" s="15">
-      <c r="B19" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-29</t>
-        </is>
-      </c>
-      <c r="C19" s="49" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D19" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E19" s="49" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F19" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1" s="15">
-      <c r="B20" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C20" s="48" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D20" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E20" s="48" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-04-30 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F20" s="48" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-04-30-day-4.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1" s="15">
-      <c r="B21" s="49" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C21" s="49" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D21" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E21" s="49" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F21" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="36" customHeight="1" s="15">
-      <c r="B22" s="48" t="inlineStr">
-        <is>
-          <t>2026-04-30</t>
-        </is>
-      </c>
-      <c r="C22" s="48" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D22" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E22" s="48" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F22" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="36" customHeight="1" s="15">
-      <c r="B23" s="49" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C23" s="49" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D23" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E23" s="49" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-01 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F23" s="49" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-05-01-day-5.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="36" customHeight="1" s="15">
-      <c r="B24" s="48" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C24" s="48" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D24" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E24" s="48" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F24" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="36" customHeight="1" s="15">
-      <c r="B25" s="49" t="inlineStr">
-        <is>
-          <t>2026-05-01</t>
-        </is>
-      </c>
-      <c r="C25" s="49" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D25" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E25" s="49" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F25" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="36" customHeight="1" s="15">
-      <c r="B26" s="48" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="C26" s="48" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D26" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E26" s="48" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-02 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F26" s="48" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-05-02-day-6.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="36" customHeight="1" s="15">
-      <c r="B27" s="49" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="C27" s="49" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D27" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E27" s="49" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F27" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="36" customHeight="1" s="15">
-      <c r="B28" s="48" t="inlineStr">
-        <is>
-          <t>2026-05-02</t>
-        </is>
-      </c>
-      <c r="C28" s="48" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D28" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E28" s="48" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F28" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="36" customHeight="1" s="15">
-      <c r="B29" s="49" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="C29" s="49" t="inlineStr">
-        <is>
-          <t>MAIN</t>
-        </is>
-      </c>
-      <c r="D29" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E29" s="49" t="inlineStr">
-        <is>
-          <t>Stop hook didn't write a token-savings.jsonl row on 2026-05-03 (likely session cleanly closed without Stop event, OR session crossed midnight UTC)</t>
-        </is>
-      </c>
-      <c r="F29" s="49" t="inlineStr">
-        <is>
-          <t>Reconstruct hours from docs/eod-reports/2026-05-03-day-7.md; tokens unrecoverable for past sessions</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="36" customHeight="1" s="15">
-      <c r="B30" s="48" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="C30" s="48" t="inlineStr">
-        <is>
-          <t>FE</t>
-        </is>
-      </c>
-      <c r="D30" s="48" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E30" s="48" t="inlineStr">
-        <is>
-          <t>FE worktree Stop hook NEVER fired (audit.jsonl absent — Bug A in token-tracking-diagnostic-2026-05-04.md)</t>
-        </is>
-      </c>
-      <c r="F30" s="48" t="inlineStr">
-        <is>
-          <t>Operator self-report from FE+1 EOD summary; followup (z) to investigate hook activation Day 9 morning</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="36" customHeight="1" s="15">
-      <c r="B31" s="49" t="inlineStr">
-        <is>
-          <t>2026-05-03</t>
-        </is>
-      </c>
-      <c r="C31" s="49" t="inlineStr">
-        <is>
-          <t>BE</t>
-        </is>
-      </c>
-      <c r="D31" s="49" t="inlineStr">
-        <is>
-          <t>All token + hours fields</t>
-        </is>
-      </c>
-      <c r="E31" s="49" t="inlineStr">
-        <is>
-          <t>BE worktree Stop hook fired through 2026-04-28 then stopped (Bug B in diagnostic doc)</t>
-        </is>
-      </c>
-      <c r="F31" s="49" t="inlineStr">
-        <is>
-          <t>Operator self-report from BE+1 EOD summary; same followup (z) as FE</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B3:F3"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="B2:F49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
@@ -12482,4 +14566,160 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8" outlineLevelRow="7"/>
+  <cols>
+    <col width="3" customWidth="1" style="15" min="1" max="1"/>
+    <col width="14" customWidth="1" style="15" min="2" max="2"/>
+    <col width="12" customWidth="1" style="15" min="3" max="3"/>
+    <col width="22" customWidth="1" style="15" min="4" max="4"/>
+    <col width="12" customWidth="1" style="15" min="5" max="6"/>
+    <col width="42" customWidth="1" style="15" min="7" max="7"/>
+    <col width="50" customWidth="1" style="15" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="31.5" customHeight="1" s="15">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Idea Confirmation — Session Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="27.75" customHeight="1" s="15">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1 — vision, market research, problem statement, solution design, mockups, competitive analysis, flow diagrams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="15">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Timing</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Evidence / Theme</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>What I Did</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19.5" customHeight="1" s="15">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>10:28 PM – 10:28 PM</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>QA_Nexus_Brainstorm.md</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="19.5" customHeight="1" s="15">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>8:22 PM – 11:30 PM</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>QA_Roles_Documents_Reference_Guide.md · QA_Nexus_Platform_Vision.md · problem-landscape.drawio</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="15">
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="n"/>
+      <c r="D8" s="54" t="n"/>
+      <c r="E8" s="13">
+        <f>SUM(E6:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="14">
+        <f>SUM(F6:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="54" t="n"/>
+      <c r="H8" s="54" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore(observability): day-17 m3 close backfill — work-log + sessions-stream
day-17 main row added to all sessions sheet (10:00 ist start →
22:30 ist end, 12.5 hr, 28 files, development phase, theme
"day-17 m3 close ceremony + 4-pr auth saga + m3 close pr").
phase sheet "development" row 20; chrono "all sessions" row 67.
grand total =sum auto-extended.

token sessions rebuilt from .claude/token-savings.jsonl
(31 sessions / 9 with data, after rebuild).

sessions-stream.jsonl already has 1 day-17 main entry from stop
hook auto-append; this commit captures the latest entry.

step 7 of m3 close ceremony resolved (was deferred to follow-up
pr to keep #141 review surface focused).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4845,7 +4845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H20"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5314,24 +5314,55 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="37" t="inlineStr">
+    <row r="20" ht="64" customHeight="1" s="15">
+      <c r="B20" s="100" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C20" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D20" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 10:30 PM</t>
+        </is>
+      </c>
+      <c r="E20" s="103" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F20" s="101" t="n">
+        <v>28</v>
+      </c>
+      <c r="G20" s="102" t="inlineStr">
+        <is>
+          <t>Day-17 M3 close ceremony + 4-PR auth saga + M3 close PR</t>
+        </is>
+      </c>
+      <c r="H20" s="102" t="inlineStr">
+        <is>
+          <t>M3 OFFICIALLY CLOSED at 22:55 IST. 13 PRs merged today (#129 #130 #131 #132 #133 #134 #137 #138 #139 #135 #136 #141 #142). 9-PR BetterAuth fix chain finally complete (Day-15 5-PR + Day-17 4-PR saga: #137 Gmail prefetch intermediate confirm page, #138 zod scoped override for @better-auth/core + 4-layer proof, #139 drop /auth/ prefix in sendMagicLink URL, plus BetterAuth &gt;=1.6.11 hardcoded single-use atomic consumption discovery). Magic-link end-to-end confirmed green by Yogesh through Gmail at 21:00 IST. F19 Run Console + AdminShell canonical realignment landed. CLAUDE.md amended with Hard Rule 14 (AdminShell F19-canonical) + Hard Rule 16 NEW (canonical-first port workflow 8 steps). 12 close-ceremony artifacts shipped in PR #141 + PR #142 (M2+M3 retro). Tag m3-closed-2026-05-13 anchored at SHA a98797b (#139 — auth-chain-complete commit). 52 PRs across M3 sprint (6 calendar days / ~3.6 working days).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="13">
-        <f>SUM(E6:E19)</f>
+      <c r="C21" s="54" t="n"/>
+      <c r="D21" s="54" t="n"/>
+      <c r="E21" s="13">
+        <f>SUM(E6:E20)</f>
         <v/>
       </c>
-      <c r="F20" s="14">
-        <f>SUM(F6:F19)</f>
+      <c r="F21" s="14">
+        <f>SUM(F6:F20)</f>
         <v/>
       </c>
-      <c r="G20" s="54" t="n"/>
-      <c r="H20" s="54" t="n"/>
+      <c r="G21" s="54" t="n"/>
+      <c r="H21" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5563,7 +5594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7237,11 +7268,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -7250,45 +7281,45 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>60</v>
       </c>
       <c r="G29" t="n">
-        <v>654</v>
+        <v>713</v>
       </c>
       <c r="H29" t="n">
-        <v>26460478</v>
+        <v>46306825</v>
       </c>
       <c r="I29" t="n">
-        <v>2937629</v>
+        <v>4100478</v>
       </c>
       <c r="J29" t="n">
-        <v>1625660118</v>
+        <v>1588281389</v>
       </c>
       <c r="K29" t="n">
-        <v>237900</v>
+        <v>259050</v>
       </c>
       <c r="L29" t="n">
-        <v>630.9856</v>
+        <v>711.6376</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>chore/claude-rule-14-app-shell-parity</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O29" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
@@ -7299,11 +7330,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -7312,45 +7343,45 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
-        <v>670</v>
+        <v>753</v>
       </c>
       <c r="H30" t="n">
-        <v>10020222</v>
+        <v>10000776</v>
       </c>
       <c r="I30" t="n">
-        <v>1275987</v>
+        <v>1227563</v>
       </c>
       <c r="J30" t="n">
-        <v>671517086</v>
+        <v>488403924</v>
       </c>
       <c r="K30" t="n">
-        <v>243500</v>
+        <v>273850</v>
       </c>
       <c r="L30" t="n">
-        <v>258.1679</v>
+        <v>202.436</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>docs/eod-day-11-main-section</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O30" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -7361,11 +7392,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7374,47 +7405,109 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>60</v>
       </c>
       <c r="G31" t="n">
-        <v>673</v>
+        <v>756</v>
       </c>
       <c r="H31" t="n">
-        <v>39681497</v>
+        <v>45415145</v>
       </c>
       <c r="I31" t="n">
-        <v>3747928</v>
+        <v>4184424</v>
       </c>
       <c r="J31" t="n">
-        <v>1459168818</v>
+        <v>2218825186</v>
       </c>
       <c r="K31" t="n">
-        <v>245050</v>
+        <v>275400</v>
       </c>
       <c r="L31" t="n">
-        <v>642.7711</v>
+        <v>898.7018</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>docs/eod-day-11-main-section</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O31" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P31" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>17</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>60</v>
+      </c>
+      <c r="G32" t="n">
+        <v>718</v>
+      </c>
+      <c r="H32" t="n">
+        <v>32787696</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1825184</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1361049886</v>
+      </c>
+      <c r="K32" t="n">
+        <v>261100</v>
+      </c>
+      <c r="L32" t="n">
+        <v>558.6419</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>docs/m3-retro</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>15</v>
+      </c>
+      <c r="P32" t="inlineStr">
         <is>
           <t>conversation</t>
         </is>
@@ -7431,7 +7524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7577,32 +7670,63 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>2.98</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>1997</v>
+        <v>2222</v>
       </c>
       <c r="F5" t="n">
-        <v>76162197</v>
+        <v>101722746</v>
       </c>
       <c r="G5" t="n">
-        <v>7961544</v>
+        <v>9512465</v>
       </c>
       <c r="H5" t="n">
-        <v>726450</v>
+        <v>808300</v>
       </c>
       <c r="I5" t="n">
-        <v>1531.9246</v>
+        <v>1812.7754</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>718</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32787696</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1825184</v>
+      </c>
+      <c r="H6" t="n">
+        <v>261100</v>
+      </c>
+      <c r="I6" t="n">
+        <v>558.6419</v>
       </c>
     </row>
   </sheetData>
@@ -7678,31 +7802,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>20.32</v>
+        <v>21.33</v>
       </c>
       <c r="D2" t="n">
-        <v>2935</v>
+        <v>3878</v>
       </c>
       <c r="E2" t="n">
-        <v>134747468</v>
+        <v>193095713</v>
       </c>
       <c r="F2" t="n">
-        <v>13178907</v>
+        <v>16555012</v>
       </c>
       <c r="G2" t="n">
-        <v>1056000</v>
+        <v>1398950</v>
       </c>
       <c r="H2" t="n">
-        <v>2444.4979</v>
+        <v>3283.9906</v>
       </c>
       <c r="I2" t="n">
-        <v>51969</v>
+        <v>65586</v>
       </c>
       <c r="J2" t="n">
-        <v>10.22</v>
+        <v>11.66</v>
       </c>
     </row>
     <row r="3">
@@ -7712,31 +7836,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>20.32</v>
+        <v>21.33</v>
       </c>
       <c r="D3" t="n">
-        <v>2935</v>
+        <v>3878</v>
       </c>
       <c r="E3" t="n">
-        <v>134747468</v>
+        <v>193095713</v>
       </c>
       <c r="F3" t="n">
-        <v>13178907</v>
+        <v>16555012</v>
       </c>
       <c r="G3" t="n">
-        <v>1056000</v>
+        <v>1398950</v>
       </c>
       <c r="H3" t="n">
-        <v>2444.4979</v>
+        <v>3283.9906</v>
       </c>
       <c r="I3" t="n">
-        <v>51969</v>
+        <v>65586</v>
       </c>
       <c r="J3" t="n">
-        <v>10.22</v>
+        <v>11.66</v>
       </c>
     </row>
   </sheetData>
@@ -7750,7 +7874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J67"/>
+  <dimension ref="B2:J68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -9912,25 +10036,62 @@
       </c>
       <c r="J66" s="102" t="n"/>
     </row>
-    <row r="67">
-      <c r="B67" s="37" t="inlineStr">
+    <row r="67" ht="64" customHeight="1" s="15">
+      <c r="B67" s="100" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C67" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D67" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 10:30 PM</t>
+        </is>
+      </c>
+      <c r="E67" s="103" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F67" s="101" t="n">
+        <v>28</v>
+      </c>
+      <c r="G67" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H67" s="102" t="inlineStr">
+        <is>
+          <t>Day-17 M3 close ceremony + 4-PR auth saga + M3 close PR</t>
+        </is>
+      </c>
+      <c r="I67" s="102" t="inlineStr">
+        <is>
+          <t>M3 OFFICIALLY CLOSED at 22:55 IST. 13 PRs merged today (#129 #130 #131 #132 #133 #134 #137 #138 #139 #135 #136 #141 #142). 9-PR BetterAuth fix chain finally complete (Day-15 5-PR + Day-17 4-PR saga: #137 Gmail prefetch intermediate confirm page, #138 zod scoped override for @better-auth/core + 4-layer proof, #139 drop /auth/ prefix in sendMagicLink URL, plus BetterAuth &gt;=1.6.11 hardcoded single-use atomic consumption discovery). Magic-link end-to-end confirmed green by Yogesh through Gmail at 21:00 IST. F19 Run Console + AdminShell canonical realignment landed. CLAUDE.md amended with Hard Rule 14 (AdminShell F19-canonical) + Hard Rule 16 NEW (canonical-first port workflow 8 steps). 12 close-ceremony artifacts shipped in PR #141 + PR #142 (M2+M3 retro). Tag m3-closed-2026-05-13 anchored at SHA a98797b (#139 — auth-chain-complete commit). 52 PRs across M3 sprint (6 calendar days / ~3.6 working days).</t>
+        </is>
+      </c>
+      <c r="J67" s="102" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C67" s="54" t="n"/>
-      <c r="D67" s="54" t="n"/>
-      <c r="E67" s="72">
-        <f>SUM(E6:E66)</f>
+      <c r="C68" s="54" t="n"/>
+      <c r="D68" s="54" t="n"/>
+      <c r="E68" s="72">
+        <f>SUM(E6:E67)</f>
         <v/>
       </c>
-      <c r="F67" s="14">
-        <f>SUM(F6:F66)</f>
+      <c r="F68" s="14">
+        <f>SUM(F6:F67)</f>
         <v/>
       </c>
-      <c r="G67" s="54" t="n"/>
-      <c r="H67" s="54" t="n"/>
-      <c r="I67" s="54" t="n"/>
+      <c r="G68" s="54" t="n"/>
+      <c r="H68" s="54" t="n"/>
+      <c r="I68" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore(observability): day-17 m3 close backfill — work-log + sessions-stream (#143)
day-17 main row added to all sessions sheet (10:00 ist start →
22:30 ist end, 12.5 hr, 28 files, development phase, theme
"day-17 m3 close ceremony + 4-pr auth saga + m3 close pr").
phase sheet "development" row 20; chrono "all sessions" row 67.
grand total =sum auto-extended.

token sessions rebuilt from .claude/token-savings.jsonl
(31 sessions / 9 with data, after rebuild).

sessions-stream.jsonl already has 1 day-17 main entry from stop
hook auto-append; this commit captures the latest entry.

step 7 of m3 close ceremony resolved (was deferred to follow-up
pr to keep #141 review surface focused).

Co-authored-by: Yogesh Mohite <yogeshmohite@admins-MacBook-Air.local>
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4845,7 +4845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H20"/>
+  <dimension ref="B2:H21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5314,24 +5314,55 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="37" t="inlineStr">
+    <row r="20" ht="64" customHeight="1" s="15">
+      <c r="B20" s="100" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C20" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D20" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 10:30 PM</t>
+        </is>
+      </c>
+      <c r="E20" s="103" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F20" s="101" t="n">
+        <v>28</v>
+      </c>
+      <c r="G20" s="102" t="inlineStr">
+        <is>
+          <t>Day-17 M3 close ceremony + 4-PR auth saga + M3 close PR</t>
+        </is>
+      </c>
+      <c r="H20" s="102" t="inlineStr">
+        <is>
+          <t>M3 OFFICIALLY CLOSED at 22:55 IST. 13 PRs merged today (#129 #130 #131 #132 #133 #134 #137 #138 #139 #135 #136 #141 #142). 9-PR BetterAuth fix chain finally complete (Day-15 5-PR + Day-17 4-PR saga: #137 Gmail prefetch intermediate confirm page, #138 zod scoped override for @better-auth/core + 4-layer proof, #139 drop /auth/ prefix in sendMagicLink URL, plus BetterAuth &gt;=1.6.11 hardcoded single-use atomic consumption discovery). Magic-link end-to-end confirmed green by Yogesh through Gmail at 21:00 IST. F19 Run Console + AdminShell canonical realignment landed. CLAUDE.md amended with Hard Rule 14 (AdminShell F19-canonical) + Hard Rule 16 NEW (canonical-first port workflow 8 steps). 12 close-ceremony artifacts shipped in PR #141 + PR #142 (M2+M3 retro). Tag m3-closed-2026-05-13 anchored at SHA a98797b (#139 — auth-chain-complete commit). 52 PRs across M3 sprint (6 calendar days / ~3.6 working days).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="54" t="n"/>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="13">
-        <f>SUM(E6:E19)</f>
+      <c r="C21" s="54" t="n"/>
+      <c r="D21" s="54" t="n"/>
+      <c r="E21" s="13">
+        <f>SUM(E6:E20)</f>
         <v/>
       </c>
-      <c r="F20" s="14">
-        <f>SUM(F6:F19)</f>
+      <c r="F21" s="14">
+        <f>SUM(F6:F20)</f>
         <v/>
       </c>
-      <c r="G20" s="54" t="n"/>
-      <c r="H20" s="54" t="n"/>
+      <c r="G21" s="54" t="n"/>
+      <c r="H21" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5563,7 +5594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:P32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7237,11 +7268,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -7250,45 +7281,45 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>10:06</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>11:06</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="F29" t="n">
         <v>60</v>
       </c>
       <c r="G29" t="n">
-        <v>654</v>
+        <v>713</v>
       </c>
       <c r="H29" t="n">
-        <v>26460478</v>
+        <v>46306825</v>
       </c>
       <c r="I29" t="n">
-        <v>2937629</v>
+        <v>4100478</v>
       </c>
       <c r="J29" t="n">
-        <v>1625660118</v>
+        <v>1588281389</v>
       </c>
       <c r="K29" t="n">
-        <v>237900</v>
+        <v>259050</v>
       </c>
       <c r="L29" t="n">
-        <v>630.9856</v>
+        <v>711.6376</v>
       </c>
       <c r="M29" t="n">
         <v>0</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>chore/claude-rule-14-app-shell-parity</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O29" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
@@ -7299,11 +7330,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -7312,45 +7343,45 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
-        <v>670</v>
+        <v>753</v>
       </c>
       <c r="H30" t="n">
-        <v>10020222</v>
+        <v>10000776</v>
       </c>
       <c r="I30" t="n">
-        <v>1275987</v>
+        <v>1227563</v>
       </c>
       <c r="J30" t="n">
-        <v>671517086</v>
+        <v>488403924</v>
       </c>
       <c r="K30" t="n">
-        <v>243500</v>
+        <v>273850</v>
       </c>
       <c r="L30" t="n">
-        <v>258.1679</v>
+        <v>202.436</v>
       </c>
       <c r="M30" t="n">
         <v>0</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>docs/eod-day-11-main-section</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O30" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P30" t="inlineStr">
         <is>
@@ -7361,11 +7392,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7374,47 +7405,109 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>11:11</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>60</v>
       </c>
       <c r="G31" t="n">
-        <v>673</v>
+        <v>756</v>
       </c>
       <c r="H31" t="n">
-        <v>39681497</v>
+        <v>45415145</v>
       </c>
       <c r="I31" t="n">
-        <v>3747928</v>
+        <v>4184424</v>
       </c>
       <c r="J31" t="n">
-        <v>1459168818</v>
+        <v>2218825186</v>
       </c>
       <c r="K31" t="n">
-        <v>245050</v>
+        <v>275400</v>
       </c>
       <c r="L31" t="n">
-        <v>642.7711</v>
+        <v>898.7018</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>docs/eod-day-11-main-section</t>
+          <t>main</t>
         </is>
       </c>
       <c r="O31" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P31" t="inlineStr">
+        <is>
+          <t>conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>17</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>60</v>
+      </c>
+      <c r="G32" t="n">
+        <v>718</v>
+      </c>
+      <c r="H32" t="n">
+        <v>32787696</v>
+      </c>
+      <c r="I32" t="n">
+        <v>1825184</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1361049886</v>
+      </c>
+      <c r="K32" t="n">
+        <v>261100</v>
+      </c>
+      <c r="L32" t="n">
+        <v>558.6419</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>docs/m3-retro</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>15</v>
+      </c>
+      <c r="P32" t="inlineStr">
         <is>
           <t>conversation</t>
         </is>
@@ -7431,7 +7524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7577,32 +7670,63 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
         <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>2.98</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>1997</v>
+        <v>2222</v>
       </c>
       <c r="F5" t="n">
-        <v>76162197</v>
+        <v>101722746</v>
       </c>
       <c r="G5" t="n">
-        <v>7961544</v>
+        <v>9512465</v>
       </c>
       <c r="H5" t="n">
-        <v>726450</v>
+        <v>808300</v>
       </c>
       <c r="I5" t="n">
-        <v>1531.9246</v>
+        <v>1812.7754</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>17</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>718</v>
+      </c>
+      <c r="F6" t="n">
+        <v>32787696</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1825184</v>
+      </c>
+      <c r="H6" t="n">
+        <v>261100</v>
+      </c>
+      <c r="I6" t="n">
+        <v>558.6419</v>
       </c>
     </row>
   </sheetData>
@@ -7678,31 +7802,31 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="n">
-        <v>20.32</v>
+        <v>21.33</v>
       </c>
       <c r="D2" t="n">
-        <v>2935</v>
+        <v>3878</v>
       </c>
       <c r="E2" t="n">
-        <v>134747468</v>
+        <v>193095713</v>
       </c>
       <c r="F2" t="n">
-        <v>13178907</v>
+        <v>16555012</v>
       </c>
       <c r="G2" t="n">
-        <v>1056000</v>
+        <v>1398950</v>
       </c>
       <c r="H2" t="n">
-        <v>2444.4979</v>
+        <v>3283.9906</v>
       </c>
       <c r="I2" t="n">
-        <v>51969</v>
+        <v>65586</v>
       </c>
       <c r="J2" t="n">
-        <v>10.22</v>
+        <v>11.66</v>
       </c>
     </row>
     <row r="3">
@@ -7712,31 +7836,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>20.32</v>
+        <v>21.33</v>
       </c>
       <c r="D3" t="n">
-        <v>2935</v>
+        <v>3878</v>
       </c>
       <c r="E3" t="n">
-        <v>134747468</v>
+        <v>193095713</v>
       </c>
       <c r="F3" t="n">
-        <v>13178907</v>
+        <v>16555012</v>
       </c>
       <c r="G3" t="n">
-        <v>1056000</v>
+        <v>1398950</v>
       </c>
       <c r="H3" t="n">
-        <v>2444.4979</v>
+        <v>3283.9906</v>
       </c>
       <c r="I3" t="n">
-        <v>51969</v>
+        <v>65586</v>
       </c>
       <c r="J3" t="n">
-        <v>10.22</v>
+        <v>11.66</v>
       </c>
     </row>
   </sheetData>
@@ -7750,7 +7874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J67"/>
+  <dimension ref="B2:J68"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -9912,25 +10036,62 @@
       </c>
       <c r="J66" s="102" t="n"/>
     </row>
-    <row r="67">
-      <c r="B67" s="37" t="inlineStr">
+    <row r="67" ht="64" customHeight="1" s="15">
+      <c r="B67" s="100" t="n">
+        <v>46155</v>
+      </c>
+      <c r="C67" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D67" s="102" t="inlineStr">
+        <is>
+          <t>10:00 AM – 10:30 PM</t>
+        </is>
+      </c>
+      <c r="E67" s="103" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F67" s="101" t="n">
+        <v>28</v>
+      </c>
+      <c r="G67" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H67" s="102" t="inlineStr">
+        <is>
+          <t>Day-17 M3 close ceremony + 4-PR auth saga + M3 close PR</t>
+        </is>
+      </c>
+      <c r="I67" s="102" t="inlineStr">
+        <is>
+          <t>M3 OFFICIALLY CLOSED at 22:55 IST. 13 PRs merged today (#129 #130 #131 #132 #133 #134 #137 #138 #139 #135 #136 #141 #142). 9-PR BetterAuth fix chain finally complete (Day-15 5-PR + Day-17 4-PR saga: #137 Gmail prefetch intermediate confirm page, #138 zod scoped override for @better-auth/core + 4-layer proof, #139 drop /auth/ prefix in sendMagicLink URL, plus BetterAuth &gt;=1.6.11 hardcoded single-use atomic consumption discovery). Magic-link end-to-end confirmed green by Yogesh through Gmail at 21:00 IST. F19 Run Console + AdminShell canonical realignment landed. CLAUDE.md amended with Hard Rule 14 (AdminShell F19-canonical) + Hard Rule 16 NEW (canonical-first port workflow 8 steps). 12 close-ceremony artifacts shipped in PR #141 + PR #142 (M2+M3 retro). Tag m3-closed-2026-05-13 anchored at SHA a98797b (#139 — auth-chain-complete commit). 52 PRs across M3 sprint (6 calendar days / ~3.6 working days).</t>
+        </is>
+      </c>
+      <c r="J67" s="102" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C67" s="54" t="n"/>
-      <c r="D67" s="54" t="n"/>
-      <c r="E67" s="72">
-        <f>SUM(E6:E66)</f>
+      <c r="C68" s="54" t="n"/>
+      <c r="D68" s="54" t="n"/>
+      <c r="E68" s="72">
+        <f>SUM(E6:E67)</f>
         <v/>
       </c>
-      <c r="F67" s="14">
-        <f>SUM(F6:F66)</f>
+      <c r="F68" s="14">
+        <f>SUM(F6:F67)</f>
         <v/>
       </c>
-      <c r="G67" s="54" t="n"/>
-      <c r="H67" s="54" t="n"/>
-      <c r="I67" s="54" t="n"/>
+      <c r="G68" s="54" t="n"/>
+      <c r="H68" s="54" t="n"/>
+      <c r="I68" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs(m4): close ceremony — EOD amend + retro + work log + followups
M4 CLOSED at 19:00 IST Sun 2026-05-17 per Yogesh ceremony brief.

PR #169 (F20 Run Results re-port) MERGED at 14:49:53Z — visual gate
PASSED at 1970a8a in 7 rounds.

Ceremony artifacts:
1. EOD amendment with M4 close section + ship state + 0 Hard Rule 11
   fires Day-20 + Day-21 priority queue
2. NEW M4 retro FE perspective memo (docs/m4/retro/fe-day-20-perspective.md)
   3-section: what worked / what hurt / what's next
3. Work log Day-20 entry (xlsx row 21 Development / 68 chrono — 6 hr
   15:00-21:00 IST)
4. 6 new followups (m)-(r): F19 P0 · F22 P1 · Kimi HIGH stretch ·
   skill v2.2 escalation · prettier housekeeping · 5-7 round refinement

Memory: feedback_f21 + feedback_f20 both indexed.
PR #171 stays [HOLD] for Day-21 docs wave.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4845,7 +4845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4857,6 +4857,7 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4871,6 +4872,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5345,24 +5347,55 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="37" t="inlineStr">
+    <row r="21" ht="64" customHeight="1" s="15">
+      <c r="B21" s="100" t="n">
+        <v>46159</v>
+      </c>
+      <c r="C21" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D21" s="102" t="inlineStr">
+        <is>
+          <t>3:00 PM – 9:00 PM</t>
+        </is>
+      </c>
+      <c r="E21" s="103" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="101" t="n">
+        <v>17</v>
+      </c>
+      <c r="G21" s="102" t="inlineStr">
+        <is>
+          <t>F20 Run Results re-port via frame-port skill v2.1.2 [M4 close]</t>
+        </is>
+      </c>
+      <c r="H21" s="102" t="inlineStr">
+        <is>
+          <t>Day-20 M4 close ceremony. F20 Run Results PR #169 visual gate PASSED at 1970a8a in 7 rounds. 7-step skill workflow validated. 24 canonical fidelity fixes. Day-18 audit recovery: 10.1% Rule 17 -&gt; 0%. 5 reusable TSX patterns archived for Day-21 (rs-stats horizontal-scroll, 3-row button stack, mobile right-rail stacking, header layout, code-block styling). PR #169 MERGED at 14:49:53Z. M4 CLOSED at 19:00 IST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C21" s="54" t="n"/>
-      <c r="D21" s="54" t="n"/>
-      <c r="E21" s="13">
-        <f>SUM(E6:E20)</f>
+      <c r="C22" s="54" t="n"/>
+      <c r="D22" s="54" t="n"/>
+      <c r="E22" s="13">
+        <f>SUM(E6:E21)</f>
         <v/>
       </c>
-      <c r="F21" s="14">
-        <f>SUM(F6:F20)</f>
+      <c r="F22" s="14">
+        <f>SUM(F6:F21)</f>
         <v/>
       </c>
-      <c r="G21" s="54" t="n"/>
-      <c r="H21" s="54" t="n"/>
+      <c r="G22" s="54" t="n"/>
+      <c r="H22" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5727,7 +5760,6 @@
       <c r="M2" t="n">
         <v>0</v>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -5785,7 +5817,6 @@
       <c r="M3" t="n">
         <v>0</v>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>0</v>
       </c>
@@ -5843,7 +5874,6 @@
       <c r="M4" t="n">
         <v>0</v>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0</v>
       </c>
@@ -5901,7 +5931,6 @@
       <c r="M5" t="n">
         <v>0</v>
       </c>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
         <v>0</v>
       </c>
@@ -5959,7 +5988,6 @@
       <c r="M6" t="n">
         <v>0</v>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
         <v>0</v>
       </c>
@@ -6079,7 +6107,6 @@
       <c r="M8" t="n">
         <v>0</v>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>0</v>
       </c>
@@ -6137,7 +6164,6 @@
       <c r="M9" t="n">
         <v>0</v>
       </c>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -6381,7 +6407,6 @@
       <c r="M13" t="n">
         <v>0</v>
       </c>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
         <v>0</v>
       </c>
@@ -6439,7 +6464,6 @@
       <c r="M14" t="n">
         <v>0</v>
       </c>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
         <v>0</v>
       </c>
@@ -6497,7 +6521,6 @@
       <c r="M15" t="n">
         <v>0</v>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
         <v>0</v>
       </c>
@@ -6555,7 +6578,6 @@
       <c r="M16" t="n">
         <v>0</v>
       </c>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
         <v>0</v>
       </c>
@@ -6613,7 +6635,6 @@
       <c r="M17" t="n">
         <v>0</v>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>0</v>
       </c>
@@ -6671,7 +6692,6 @@
       <c r="M18" t="n">
         <v>0</v>
       </c>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
         <v>0</v>
       </c>
@@ -6729,7 +6749,6 @@
       <c r="M19" t="n">
         <v>0</v>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>0</v>
       </c>
@@ -6787,7 +6806,6 @@
       <c r="M20" t="n">
         <v>0</v>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
         <v>0</v>
       </c>
@@ -6845,7 +6863,6 @@
       <c r="M21" t="n">
         <v>0</v>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>0</v>
       </c>
@@ -6903,7 +6920,6 @@
       <c r="M22" t="n">
         <v>0</v>
       </c>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
         <v>0</v>
       </c>
@@ -6961,7 +6977,6 @@
       <c r="M23" t="n">
         <v>0</v>
       </c>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
         <v>0</v>
       </c>
@@ -7019,7 +7034,6 @@
       <c r="M24" t="n">
         <v>0</v>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
         <v>0</v>
       </c>
@@ -7077,7 +7091,6 @@
       <c r="M25" t="n">
         <v>0</v>
       </c>
-      <c r="N25" t="inlineStr"/>
       <c r="O25" t="n">
         <v>0</v>
       </c>
@@ -7135,7 +7148,6 @@
       <c r="M26" t="n">
         <v>0</v>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
         <v>0</v>
       </c>
@@ -7193,7 +7205,6 @@
       <c r="M27" t="n">
         <v>0</v>
       </c>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
         <v>0</v>
       </c>
@@ -7874,7 +7885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -7889,6 +7900,7 @@
     <col width="50" customWidth="1" style="15" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -7903,6 +7915,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -10073,25 +10086,62 @@
       </c>
       <c r="J67" s="102" t="n"/>
     </row>
-    <row r="68">
-      <c r="B68" s="37" t="inlineStr">
+    <row r="68" ht="64" customHeight="1" s="15">
+      <c r="B68" s="100" t="n">
+        <v>46159</v>
+      </c>
+      <c r="C68" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D68" s="102" t="inlineStr">
+        <is>
+          <t>3:00 PM – 9:00 PM</t>
+        </is>
+      </c>
+      <c r="E68" s="103" t="n">
+        <v>6</v>
+      </c>
+      <c r="F68" s="101" t="n">
+        <v>17</v>
+      </c>
+      <c r="G68" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H68" s="102" t="inlineStr">
+        <is>
+          <t>F20 Run Results re-port via frame-port skill v2.1.2 [M4 close]</t>
+        </is>
+      </c>
+      <c r="I68" s="102" t="inlineStr">
+        <is>
+          <t>Day-20 M4 close ceremony. F20 Run Results PR #169 visual gate PASSED at 1970a8a in 7 rounds. 7-step skill workflow validated. 24 canonical fidelity fixes. Day-18 audit recovery: 10.1% Rule 17 -&gt; 0%. 5 reusable TSX patterns archived for Day-21 (rs-stats horizontal-scroll, 3-row button stack, mobile right-rail stacking, header layout, code-block styling). PR #169 MERGED at 14:49:53Z. M4 CLOSED at 19:00 IST.</t>
+        </is>
+      </c>
+      <c r="J68" s="102" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C68" s="54" t="n"/>
-      <c r="D68" s="54" t="n"/>
-      <c r="E68" s="72">
-        <f>SUM(E6:E67)</f>
+      <c r="C69" s="54" t="n"/>
+      <c r="D69" s="54" t="n"/>
+      <c r="E69" s="72">
+        <f>SUM(E6:E68)</f>
         <v/>
       </c>
-      <c r="F68" s="14">
-        <f>SUM(F6:F67)</f>
+      <c r="F69" s="14">
+        <f>SUM(F6:F68)</f>
         <v/>
       </c>
-      <c r="G68" s="54" t="n"/>
-      <c r="H68" s="54" t="n"/>
-      <c r="I68" s="54" t="n"/>
+      <c r="G69" s="54" t="n"/>
+      <c r="H69" s="54" t="n"/>
+      <c r="I69" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs(eod): post day-24 main report + work-log day-23+24 backfill
day-24 wrote m5-friday-close-plan + close-report skeleton (3 plan
amendments: cascade simplified flat-base / risk-4 resolution /
saturday-wave checklist).

F25 PR #197 first bundle-workflow PASS at 16:30 IST (0% divergence).
F19 PR #198 [PARTIAL] steps 1-2 commit (day-25 resumes step 4 zero
re-extraction cost).

ADR-022 gate deferred day-25 PM; two-tier m5 close definition
ratified (tier-1 fri-binding, tier-2 sat-reserve-allowance for
F26+F28 GOVERN admin frames).

work-log rows: day-23 (7h) + day-24 (7.5h) backfilled via
update-work-log.py.

7 lessons-learned items captured in §7 including bundle-workflow
frame-specific quality + pre-stage scaffold pattern (3x validated).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4845,7 +4845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5378,24 +5378,86 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="37" t="inlineStr">
+    <row r="22" ht="64" customHeight="1" s="15">
+      <c r="B22" s="100" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C22" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E22" s="103" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" s="102" t="inlineStr">
+        <is>
+          <t>ADR-021 ratification + ADR-022 candidate refined + F22 bundle REJECTION cascade</t>
+        </is>
+      </c>
+      <c r="H22" s="102" t="inlineStr">
+        <is>
+          <t>Day-23 ratified ADR-021 via offline PR comment; refined ADR-022 candidate twice; F22 bundle REJECTED 30-50% divergence; v2-HTML re-port via Rule 15+skill v2.2 PASSED 17:25 IST; 5 cascade amendments propagated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="64" customHeight="1" s="15">
+      <c r="B23" s="100" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C23" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D23" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E23" s="103" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F23" s="101" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="102" t="inlineStr">
+        <is>
+          <t>M5 Friday close plan + F25 first bundle-workflow success + F19 PARTIAL</t>
+        </is>
+      </c>
+      <c r="H23" s="102" t="inlineStr">
+        <is>
+          <t>Day-24 wrote m5-friday-close-plan + close-report skeleton; 3 plan amendments (cascade simplified flat-base / Risk-4 resolution / Saturday-wave checklist); F25 PR #197 first bundle-workflow PASS at 16:30 IST; F19 PR #198 [PARTIAL] Steps 1-2 commit (Day-25 resumes Step 4); ADR-022 gate deferred Day-25 PM; two-tier M5 close definition Tier-1/Tier-2 ratified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="54" t="n"/>
-      <c r="D22" s="54" t="n"/>
-      <c r="E22" s="13">
-        <f>SUM(E6:E21)</f>
+      <c r="C24" s="54" t="n"/>
+      <c r="D24" s="54" t="n"/>
+      <c r="E24" s="13">
+        <f>SUM(E6:E23)</f>
         <v/>
       </c>
-      <c r="F22" s="14">
-        <f>SUM(F6:F21)</f>
+      <c r="F24" s="14">
+        <f>SUM(F6:F23)</f>
         <v/>
       </c>
-      <c r="G22" s="54" t="n"/>
-      <c r="H22" s="54" t="n"/>
+      <c r="G24" s="54" t="n"/>
+      <c r="H24" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7885,7 +7947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -10123,25 +10185,99 @@
       </c>
       <c r="J68" s="102" t="n"/>
     </row>
-    <row r="69">
-      <c r="B69" s="37" t="inlineStr">
+    <row r="69" ht="64" customHeight="1" s="15">
+      <c r="B69" s="100" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C69" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D69" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E69" s="103" t="n">
+        <v>7</v>
+      </c>
+      <c r="F69" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G69" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H69" s="102" t="inlineStr">
+        <is>
+          <t>ADR-021 ratification + ADR-022 candidate refined + F22 bundle REJECTION cascade</t>
+        </is>
+      </c>
+      <c r="I69" s="102" t="inlineStr">
+        <is>
+          <t>Day-23 ratified ADR-021 via offline PR comment; refined ADR-022 candidate twice; F22 bundle REJECTED 30-50% divergence; v2-HTML re-port via Rule 15+skill v2.2 PASSED 17:25 IST; 5 cascade amendments propagated.</t>
+        </is>
+      </c>
+      <c r="J69" s="102" t="n"/>
+    </row>
+    <row r="70" ht="64" customHeight="1" s="15">
+      <c r="B70" s="100" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C70" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D70" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E70" s="103" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F70" s="101" t="n">
+        <v>6</v>
+      </c>
+      <c r="G70" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H70" s="102" t="inlineStr">
+        <is>
+          <t>M5 Friday close plan + F25 first bundle-workflow success + F19 PARTIAL</t>
+        </is>
+      </c>
+      <c r="I70" s="102" t="inlineStr">
+        <is>
+          <t>Day-24 wrote m5-friday-close-plan + close-report skeleton; 3 plan amendments (cascade simplified flat-base / Risk-4 resolution / Saturday-wave checklist); F25 PR #197 first bundle-workflow PASS at 16:30 IST; F19 PR #198 [PARTIAL] Steps 1-2 commit (Day-25 resumes Step 4); ADR-022 gate deferred Day-25 PM; two-tier M5 close definition Tier-1/Tier-2 ratified.</t>
+        </is>
+      </c>
+      <c r="J70" s="102" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C69" s="54" t="n"/>
-      <c r="D69" s="54" t="n"/>
-      <c r="E69" s="72">
-        <f>SUM(E6:E68)</f>
+      <c r="C71" s="54" t="n"/>
+      <c r="D71" s="54" t="n"/>
+      <c r="E71" s="72">
+        <f>SUM(E6:E70)</f>
         <v/>
       </c>
-      <c r="F69" s="14">
-        <f>SUM(F6:F68)</f>
+      <c r="F71" s="14">
+        <f>SUM(F6:F70)</f>
         <v/>
       </c>
-      <c r="G69" s="54" t="n"/>
-      <c r="H69" s="54" t="n"/>
-      <c r="I69" s="54" t="n"/>
+      <c r="G71" s="54" t="n"/>
+      <c r="H71" s="54" t="n"/>
+      <c r="I71" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
docs(eod): post day-24 main report + work-log day-23+24 backfill (#200)
day-24 wrote m5-friday-close-plan + close-report skeleton (3 plan
amendments: cascade simplified flat-base / risk-4 resolution /
saturday-wave checklist).

F25 PR #197 first bundle-workflow PASS at 16:30 IST (0% divergence).
F19 PR #198 [PARTIAL] steps 1-2 commit (day-25 resumes step 4 zero
re-extraction cost).

ADR-022 gate deferred day-25 PM; two-tier m5 close definition
ratified (tier-1 fri-binding, tier-2 sat-reserve-allowance for
F26+F28 GOVERN admin frames).

work-log rows: day-23 (7h) + day-24 (7.5h) backfilled via
update-work-log.py.

7 lessons-learned items captured in §7 including bundle-workflow
frame-specific quality + pre-stage scaffold pattern (3x validated).

Co-authored-by: Yogesh Mohite <yogeshmohite@admins-MacBook-Air.local>
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4845,7 +4845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -5378,24 +5378,86 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="37" t="inlineStr">
+    <row r="22" ht="64" customHeight="1" s="15">
+      <c r="B22" s="100" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C22" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E22" s="103" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G22" s="102" t="inlineStr">
+        <is>
+          <t>ADR-021 ratification + ADR-022 candidate refined + F22 bundle REJECTION cascade</t>
+        </is>
+      </c>
+      <c r="H22" s="102" t="inlineStr">
+        <is>
+          <t>Day-23 ratified ADR-021 via offline PR comment; refined ADR-022 candidate twice; F22 bundle REJECTED 30-50% divergence; v2-HTML re-port via Rule 15+skill v2.2 PASSED 17:25 IST; 5 cascade amendments propagated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="64" customHeight="1" s="15">
+      <c r="B23" s="100" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C23" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D23" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E23" s="103" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F23" s="101" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" s="102" t="inlineStr">
+        <is>
+          <t>M5 Friday close plan + F25 first bundle-workflow success + F19 PARTIAL</t>
+        </is>
+      </c>
+      <c r="H23" s="102" t="inlineStr">
+        <is>
+          <t>Day-24 wrote m5-friday-close-plan + close-report skeleton; 3 plan amendments (cascade simplified flat-base / Risk-4 resolution / Saturday-wave checklist); F25 PR #197 first bundle-workflow PASS at 16:30 IST; F19 PR #198 [PARTIAL] Steps 1-2 commit (Day-25 resumes Step 4); ADR-022 gate deferred Day-25 PM; two-tier M5 close definition Tier-1/Tier-2 ratified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="54" t="n"/>
-      <c r="D22" s="54" t="n"/>
-      <c r="E22" s="13">
-        <f>SUM(E6:E21)</f>
+      <c r="C24" s="54" t="n"/>
+      <c r="D24" s="54" t="n"/>
+      <c r="E24" s="13">
+        <f>SUM(E6:E23)</f>
         <v/>
       </c>
-      <c r="F22" s="14">
-        <f>SUM(F6:F21)</f>
+      <c r="F24" s="14">
+        <f>SUM(F6:F23)</f>
         <v/>
       </c>
-      <c r="G22" s="54" t="n"/>
-      <c r="H22" s="54" t="n"/>
+      <c r="G24" s="54" t="n"/>
+      <c r="H24" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7885,7 +7947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -10123,25 +10185,99 @@
       </c>
       <c r="J68" s="102" t="n"/>
     </row>
-    <row r="69">
-      <c r="B69" s="37" t="inlineStr">
+    <row r="69" ht="64" customHeight="1" s="15">
+      <c r="B69" s="100" t="n">
+        <v>46162</v>
+      </c>
+      <c r="C69" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D69" s="102" t="inlineStr">
+        <is>
+          <t>11:30 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E69" s="103" t="n">
+        <v>7</v>
+      </c>
+      <c r="F69" s="101" t="n">
+        <v>10</v>
+      </c>
+      <c r="G69" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H69" s="102" t="inlineStr">
+        <is>
+          <t>ADR-021 ratification + ADR-022 candidate refined + F22 bundle REJECTION cascade</t>
+        </is>
+      </c>
+      <c r="I69" s="102" t="inlineStr">
+        <is>
+          <t>Day-23 ratified ADR-021 via offline PR comment; refined ADR-022 candidate twice; F22 bundle REJECTED 30-50% divergence; v2-HTML re-port via Rule 15+skill v2.2 PASSED 17:25 IST; 5 cascade amendments propagated.</t>
+        </is>
+      </c>
+      <c r="J69" s="102" t="n"/>
+    </row>
+    <row r="70" ht="64" customHeight="1" s="15">
+      <c r="B70" s="100" t="n">
+        <v>46163</v>
+      </c>
+      <c r="C70" s="101" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="D70" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 6:30 PM</t>
+        </is>
+      </c>
+      <c r="E70" s="103" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F70" s="101" t="n">
+        <v>6</v>
+      </c>
+      <c r="G70" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H70" s="102" t="inlineStr">
+        <is>
+          <t>M5 Friday close plan + F25 first bundle-workflow success + F19 PARTIAL</t>
+        </is>
+      </c>
+      <c r="I70" s="102" t="inlineStr">
+        <is>
+          <t>Day-24 wrote m5-friday-close-plan + close-report skeleton; 3 plan amendments (cascade simplified flat-base / Risk-4 resolution / Saturday-wave checklist); F25 PR #197 first bundle-workflow PASS at 16:30 IST; F19 PR #198 [PARTIAL] Steps 1-2 commit (Day-25 resumes Step 4); ADR-022 gate deferred Day-25 PM; two-tier M5 close definition Tier-1/Tier-2 ratified.</t>
+        </is>
+      </c>
+      <c r="J70" s="102" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C69" s="54" t="n"/>
-      <c r="D69" s="54" t="n"/>
-      <c r="E69" s="72">
-        <f>SUM(E6:E68)</f>
+      <c r="C71" s="54" t="n"/>
+      <c r="D71" s="54" t="n"/>
+      <c r="E71" s="72">
+        <f>SUM(E6:E70)</f>
         <v/>
       </c>
-      <c r="F69" s="14">
-        <f>SUM(F6:F68)</f>
+      <c r="F71" s="14">
+        <f>SUM(F6:F70)</f>
         <v/>
       </c>
-      <c r="G69" s="54" t="n"/>
-      <c r="H69" s="54" t="n"/>
-      <c r="I69" s="54" t="n"/>
+      <c r="G71" s="54" t="n"/>
+      <c r="H71" s="54" t="n"/>
+      <c r="I71" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore(m5): work-log day-25/28 rows + token-usage summary + retro skeleton [m5-followup]
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4152,7 +4152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4164,6 +4164,7 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4178,6 +4179,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -4683,24 +4685,55 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="37" t="inlineStr">
+    <row r="22" ht="64" customHeight="1" s="15">
+      <c r="B22" s="100" t="n">
+        <v>46169</v>
+      </c>
+      <c r="C22" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 4:00 PM</t>
+        </is>
+      </c>
+      <c r="E22" s="103" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="101" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE CLOSED — Phase A/B/D cascade (28 PRs) + AC042 PASS 64%/1.00 + tag m5-closed-2026-05-27</t>
+        </is>
+      </c>
+      <c r="H22" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE close day. MAIN orchestrated 28-PR cascade: Phase A 10 functional PRs (F22/F25/F19/F23 + ADR-022 #208 + #201/#206/#211/#214 + schema-fix #213 last after BE+1 rebase) + Phase B 17 EOD PRs (2 conflicts resolved inline: #193 memory union, #207 xlsx) + Phase D ceremony (close report to docs/m5, CHANGELOG to [M5 CORE], tag cut, release published). AC042 PASS top-2 64%/calibration 1.00/0 crashes via Plan A2 (Zod loosen + prompt calibration). F28 v2.3 Tier-2 bonus shipped (#214). F26+F27 carry to Day-29. Verify-before-act discipline held twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="54" t="n"/>
-      <c r="D22" s="54" t="n"/>
-      <c r="E22" s="13">
-        <f>SUM(E6:E21)</f>
+      <c r="C23" s="54" t="n"/>
+      <c r="D23" s="54" t="n"/>
+      <c r="E23" s="13">
+        <f>SUM(E6:E22)</f>
         <v/>
       </c>
-      <c r="F22" s="14">
-        <f>SUM(F6:F21)</f>
+      <c r="F23" s="14">
+        <f>SUM(F6:F22)</f>
         <v/>
       </c>
-      <c r="G22" s="54" t="n"/>
-      <c r="H22" s="54" t="n"/>
+      <c r="G23" s="54" t="n"/>
+      <c r="H23" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4845,7 +4878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="B2:H25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4857,7 +4890,6 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4872,7 +4904,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5440,24 +5471,55 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="37" t="inlineStr">
+    <row r="24" ht="64" customHeight="1" s="15">
+      <c r="B24" s="100" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C24" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D24" s="102" t="inlineStr">
+        <is>
+          <t>4:45 PM – 12:53 AM</t>
+        </is>
+      </c>
+      <c r="E24" s="103" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F24" s="101" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" s="102" t="inlineStr">
+        <is>
+          <t>Sun recovery — M5 cascade + F19+F23 + AC042 harness + close-report (regen, dropped in #207 xlsx conflict)</t>
+        </is>
+      </c>
+      <c r="H24" s="102" t="inlineStr">
+        <is>
+          <t>Sunday recovery session post Fri+Sat orchestrator-absence gap. MAIN: #185 rebase + m5-close-report refine + day-26 brief + orchestrator-absence memory. BE+1: cascade #189/#194/#195 + AC042 harness #201. FE+1: F19 #198 shipped + F23 #203 PARTIAL. Row regenerated Day-28 (dropped during #207 xlsx binary-conflict resolution; take-main-accumulated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C24" s="54" t="n"/>
-      <c r="D24" s="54" t="n"/>
-      <c r="E24" s="13">
-        <f>SUM(E6:E23)</f>
+      <c r="C25" s="54" t="n"/>
+      <c r="D25" s="54" t="n"/>
+      <c r="E25" s="13">
+        <f>SUM(E6:E24)</f>
         <v/>
       </c>
-      <c r="F24" s="14">
-        <f>SUM(F6:F23)</f>
+      <c r="F25" s="14">
+        <f>SUM(F6:F24)</f>
         <v/>
       </c>
-      <c r="G24" s="54" t="n"/>
-      <c r="H24" s="54" t="n"/>
+      <c r="G25" s="54" t="n"/>
+      <c r="H25" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7947,7 +8009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -10259,25 +10321,99 @@
       </c>
       <c r="J70" s="102" t="n"/>
     </row>
-    <row r="71">
-      <c r="B71" s="37" t="inlineStr">
+    <row r="71" ht="64" customHeight="1" s="15">
+      <c r="B71" s="100" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C71" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D71" s="102" t="inlineStr">
+        <is>
+          <t>4:45 PM – 12:53 AM</t>
+        </is>
+      </c>
+      <c r="E71" s="103" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F71" s="101" t="n">
+        <v>40</v>
+      </c>
+      <c r="G71" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H71" s="102" t="inlineStr">
+        <is>
+          <t>Sun recovery — M5 cascade + F19+F23 + AC042 harness + close-report (regen, dropped in #207 xlsx conflict)</t>
+        </is>
+      </c>
+      <c r="I71" s="102" t="inlineStr">
+        <is>
+          <t>Sunday recovery session post Fri+Sat orchestrator-absence gap. MAIN: #185 rebase + m5-close-report refine + day-26 brief + orchestrator-absence memory. BE+1: cascade #189/#194/#195 + AC042 harness #201. FE+1: F19 #198 shipped + F23 #203 PARTIAL. Row regenerated Day-28 (dropped during #207 xlsx binary-conflict resolution; take-main-accumulated).</t>
+        </is>
+      </c>
+      <c r="J71" s="102" t="n"/>
+    </row>
+    <row r="72" ht="64" customHeight="1" s="15">
+      <c r="B72" s="100" t="n">
+        <v>46169</v>
+      </c>
+      <c r="C72" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D72" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 4:00 PM</t>
+        </is>
+      </c>
+      <c r="E72" s="103" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" s="101" t="n">
+        <v>35</v>
+      </c>
+      <c r="G72" s="102" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="H72" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE CLOSED — Phase A/B/D cascade (28 PRs) + AC042 PASS 64%/1.00 + tag m5-closed-2026-05-27</t>
+        </is>
+      </c>
+      <c r="I72" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE close day. MAIN orchestrated 28-PR cascade: Phase A 10 functional PRs (F22/F25/F19/F23 + ADR-022 #208 + #201/#206/#211/#214 + schema-fix #213 last after BE+1 rebase) + Phase B 17 EOD PRs (2 conflicts resolved inline: #193 memory union, #207 xlsx) + Phase D ceremony (close report to docs/m5, CHANGELOG to [M5 CORE], tag cut, release published). AC042 PASS top-2 64%/calibration 1.00/0 crashes via Plan A2 (Zod loosen + prompt calibration). F28 v2.3 Tier-2 bonus shipped (#214). F26+F27 carry to Day-29. Verify-before-act discipline held twice.</t>
+        </is>
+      </c>
+      <c r="J72" s="102" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C71" s="54" t="n"/>
-      <c r="D71" s="54" t="n"/>
-      <c r="E71" s="72">
-        <f>SUM(E6:E70)</f>
+      <c r="C73" s="54" t="n"/>
+      <c r="D73" s="54" t="n"/>
+      <c r="E73" s="72">
+        <f>SUM(E6:E72)</f>
         <v/>
       </c>
-      <c r="F71" s="14">
-        <f>SUM(F6:F70)</f>
+      <c r="F73" s="14">
+        <f>SUM(F6:F72)</f>
         <v/>
       </c>
-      <c r="G71" s="54" t="n"/>
-      <c r="H71" s="54" t="n"/>
-      <c r="I71" s="54" t="n"/>
+      <c r="G73" s="54" t="n"/>
+      <c r="H73" s="54" t="n"/>
+      <c r="I73" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
chore(m5): work-log day-25/28 + token-usage summary + retro skeleton [m5-followup] (#219)
* chore(m5): work-log day-25/28 rows + token-usage summary + retro skeleton [m5-followup]

* docs(memory): m5 core close retrospective entries [m5-followup]

---------

Co-authored-by: Yogesh Mohite <yogeshmohite@admins-MacBook-Air.local>
</commit_message>
<xml_diff>
--- a/docs/observability/QA_Nexus_Work_Log.xlsx
+++ b/docs/observability/QA_Nexus_Work_Log.xlsx
@@ -4152,7 +4152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4164,6 +4164,7 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4178,6 +4179,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -4683,24 +4685,55 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="37" t="inlineStr">
+    <row r="22" ht="64" customHeight="1" s="15">
+      <c r="B22" s="100" t="n">
+        <v>46169</v>
+      </c>
+      <c r="C22" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 4:00 PM</t>
+        </is>
+      </c>
+      <c r="E22" s="103" t="n">
+        <v>5</v>
+      </c>
+      <c r="F22" s="101" t="n">
+        <v>35</v>
+      </c>
+      <c r="G22" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE CLOSED — Phase A/B/D cascade (28 PRs) + AC042 PASS 64%/1.00 + tag m5-closed-2026-05-27</t>
+        </is>
+      </c>
+      <c r="H22" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE close day. MAIN orchestrated 28-PR cascade: Phase A 10 functional PRs (F22/F25/F19/F23 + ADR-022 #208 + #201/#206/#211/#214 + schema-fix #213 last after BE+1 rebase) + Phase B 17 EOD PRs (2 conflicts resolved inline: #193 memory union, #207 xlsx) + Phase D ceremony (close report to docs/m5, CHANGELOG to [M5 CORE], tag cut, release published). AC042 PASS top-2 64%/calibration 1.00/0 crashes via Plan A2 (Zod loosen + prompt calibration). F28 v2.3 Tier-2 bonus shipped (#214). F26+F27 carry to Day-29. Verify-before-act discipline held twice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="54" t="n"/>
-      <c r="D22" s="54" t="n"/>
-      <c r="E22" s="13">
-        <f>SUM(E6:E21)</f>
+      <c r="C23" s="54" t="n"/>
+      <c r="D23" s="54" t="n"/>
+      <c r="E23" s="13">
+        <f>SUM(E6:E22)</f>
         <v/>
       </c>
-      <c r="F22" s="14">
-        <f>SUM(F6:F21)</f>
+      <c r="F23" s="14">
+        <f>SUM(F6:F22)</f>
         <v/>
       </c>
-      <c r="G22" s="54" t="n"/>
-      <c r="H22" s="54" t="n"/>
+      <c r="G23" s="54" t="n"/>
+      <c r="H23" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4845,7 +4878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="B2:H25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -4857,7 +4890,6 @@
     <col width="50" customWidth="1" style="15" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="31.5" customHeight="1" s="15">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -4872,7 +4904,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="15">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -5440,24 +5471,55 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="37" t="inlineStr">
+    <row r="24" ht="64" customHeight="1" s="15">
+      <c r="B24" s="100" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C24" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D24" s="102" t="inlineStr">
+        <is>
+          <t>4:45 PM – 12:53 AM</t>
+        </is>
+      </c>
+      <c r="E24" s="103" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F24" s="101" t="n">
+        <v>40</v>
+      </c>
+      <c r="G24" s="102" t="inlineStr">
+        <is>
+          <t>Sun recovery — M5 cascade + F19+F23 + AC042 harness + close-report (regen, dropped in #207 xlsx conflict)</t>
+        </is>
+      </c>
+      <c r="H24" s="102" t="inlineStr">
+        <is>
+          <t>Sunday recovery session post Fri+Sat orchestrator-absence gap. MAIN: #185 rebase + m5-close-report refine + day-26 brief + orchestrator-absence memory. BE+1: cascade #189/#194/#195 + AC042 harness #201. FE+1: F19 #198 shipped + F23 #203 PARTIAL. Row regenerated Day-28 (dropped during #207 xlsx binary-conflict resolution; take-main-accumulated).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C24" s="54" t="n"/>
-      <c r="D24" s="54" t="n"/>
-      <c r="E24" s="13">
-        <f>SUM(E6:E23)</f>
+      <c r="C25" s="54" t="n"/>
+      <c r="D25" s="54" t="n"/>
+      <c r="E25" s="13">
+        <f>SUM(E6:E24)</f>
         <v/>
       </c>
-      <c r="F24" s="14">
-        <f>SUM(F6:F23)</f>
+      <c r="F25" s="14">
+        <f>SUM(F6:F24)</f>
         <v/>
       </c>
-      <c r="G24" s="54" t="n"/>
-      <c r="H24" s="54" t="n"/>
+      <c r="G25" s="54" t="n"/>
+      <c r="H25" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7947,7 +8009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="15" min="1" max="1"/>
@@ -10259,25 +10321,99 @@
       </c>
       <c r="J70" s="102" t="n"/>
     </row>
-    <row r="71">
-      <c r="B71" s="37" t="inlineStr">
+    <row r="71" ht="64" customHeight="1" s="15">
+      <c r="B71" s="100" t="n">
+        <v>46166</v>
+      </c>
+      <c r="C71" s="101" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="D71" s="102" t="inlineStr">
+        <is>
+          <t>4:45 PM – 12:53 AM</t>
+        </is>
+      </c>
+      <c r="E71" s="103" t="n">
+        <v>8.130000000000001</v>
+      </c>
+      <c r="F71" s="101" t="n">
+        <v>40</v>
+      </c>
+      <c r="G71" s="102" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="H71" s="102" t="inlineStr">
+        <is>
+          <t>Sun recovery — M5 cascade + F19+F23 + AC042 harness + close-report (regen, dropped in #207 xlsx conflict)</t>
+        </is>
+      </c>
+      <c r="I71" s="102" t="inlineStr">
+        <is>
+          <t>Sunday recovery session post Fri+Sat orchestrator-absence gap. MAIN: #185 rebase + m5-close-report refine + day-26 brief + orchestrator-absence memory. BE+1: cascade #189/#194/#195 + AC042 harness #201. FE+1: F19 #198 shipped + F23 #203 PARTIAL. Row regenerated Day-28 (dropped during #207 xlsx binary-conflict resolution; take-main-accumulated).</t>
+        </is>
+      </c>
+      <c r="J71" s="102" t="n"/>
+    </row>
+    <row r="72" ht="64" customHeight="1" s="15">
+      <c r="B72" s="100" t="n">
+        <v>46169</v>
+      </c>
+      <c r="C72" s="101" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D72" s="102" t="inlineStr">
+        <is>
+          <t>11:00 AM – 4:00 PM</t>
+        </is>
+      </c>
+      <c r="E72" s="103" t="n">
+        <v>5</v>
+      </c>
+      <c r="F72" s="101" t="n">
+        <v>35</v>
+      </c>
+      <c r="G72" s="102" t="inlineStr">
+        <is>
+          <t>Milestone Planning</t>
+        </is>
+      </c>
+      <c r="H72" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE CLOSED — Phase A/B/D cascade (28 PRs) + AC042 PASS 64%/1.00 + tag m5-closed-2026-05-27</t>
+        </is>
+      </c>
+      <c r="I72" s="102" t="inlineStr">
+        <is>
+          <t>M5 CORE close day. MAIN orchestrated 28-PR cascade: Phase A 10 functional PRs (F22/F25/F19/F23 + ADR-022 #208 + #201/#206/#211/#214 + schema-fix #213 last after BE+1 rebase) + Phase B 17 EOD PRs (2 conflicts resolved inline: #193 memory union, #207 xlsx) + Phase D ceremony (close report to docs/m5, CHANGELOG to [M5 CORE], tag cut, release published). AC042 PASS top-2 64%/calibration 1.00/0 crashes via Plan A2 (Zod loosen + prompt calibration). F28 v2.3 Tier-2 bonus shipped (#214). F26+F27 carry to Day-29. Verify-before-act discipline held twice.</t>
+        </is>
+      </c>
+      <c r="J72" s="102" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="37" t="inlineStr">
         <is>
           <t>GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C71" s="54" t="n"/>
-      <c r="D71" s="54" t="n"/>
-      <c r="E71" s="72">
-        <f>SUM(E6:E70)</f>
+      <c r="C73" s="54" t="n"/>
+      <c r="D73" s="54" t="n"/>
+      <c r="E73" s="72">
+        <f>SUM(E6:E72)</f>
         <v/>
       </c>
-      <c r="F71" s="14">
-        <f>SUM(F6:F70)</f>
+      <c r="F73" s="14">
+        <f>SUM(F6:F72)</f>
         <v/>
       </c>
-      <c r="G71" s="54" t="n"/>
-      <c r="H71" s="54" t="n"/>
-      <c r="I71" s="54" t="n"/>
+      <c r="G73" s="54" t="n"/>
+      <c r="H73" s="54" t="n"/>
+      <c r="I73" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>